<commit_message>
D5 tomada: fecha límite el 4-ene-2027 (documento final listo para revisión); ejemplos de tesis UPS con cédulas fuera del repo [IA: Claude]
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/11_Planificacion/Cronograma_Tesis.xlsx
+++ b/11_Planificacion/Cronograma_Tesis.xlsx
@@ -3978,6 +3978,7 @@
         <v/>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
@@ -4396,7 +4397,11 @@
           <t>S10-02 (#47)</t>
         </is>
       </c>
-      <c r="N11" s="15" t="inlineStr"/>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>Escenario B confirmado (entrega 4-ene-2027): las tareas ✂ se mantienen</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
@@ -4622,6 +4627,7 @@
         <v/>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
@@ -5040,7 +5046,11 @@
           <t>H-01 (#48)</t>
         </is>
       </c>
-      <c r="N11" s="15" t="inlineStr"/>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>Última lectura antes de la fecha límite del lunes 4-ene-2027</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A5:N11"/>
@@ -5150,6 +5160,7 @@
         <v/>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
@@ -5278,7 +5289,11 @@
           <t>E-01 (#49)</t>
         </is>
       </c>
-      <c r="N6" s="15" t="inlineStr"/>
+      <c r="N6" s="15" t="inlineStr">
+        <is>
+          <t>FECHA LÍMITE (D5, Víctor 18-oct): el lunes 4-ene-2027 el documento final está completo y listo para la revisión de la tutora</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -6768,7 +6783,6 @@
         <v/>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
@@ -12348,7 +12362,6 @@
         <v/>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sprint 2 adelantado: caps. I (2 partes), II y III y lienzo en v0.1 con control de cambios, 7 fuentes verificadas (37), matriz v0.2, resumen del cap. I para Diego, cronograma y app actualizados (#13 #14 #15 #58) [IA: Claude]
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/11_Planificacion/Cronograma_Tesis.xlsx
+++ b/11_Planificacion/Cronograma_Tesis.xlsx
@@ -3978,7 +3978,6 @@
         <v/>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
@@ -4627,7 +4626,6 @@
         <v/>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
@@ -5160,7 +5158,6 @@
         <v/>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
@@ -12478,7 +12475,7 @@
       <c r="J6" s="22" t="n"/>
       <c r="K6" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="L6" s="15">
@@ -12492,7 +12489,7 @@
       </c>
       <c r="N6" s="15" t="inlineStr">
         <is>
-          <t>Bloque doble con: bajar a mano los PDF de la matriz (Oldroyd, Pollitt, Galan, Nyqvist, Lewis y Sauro, Auernhammer) → Claude los verifica</t>
+          <t>Bloque doble con: bajar a mano los PDF de la matriz (Oldroyd, Pollitt, Galan, Nyqvist, Lewis y Sauro, Auernhammer) → Claude los verifica · 19-oct: Cap. I parte 1 v0.1 hecha por Claude (control de cambios); Víctor revisa. PDF a mano: esta noche</t>
         </is>
       </c>
     </row>
@@ -12602,7 +12599,7 @@
       <c r="J8" s="22" t="n"/>
       <c r="K8" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="L8" s="15">
@@ -12616,7 +12613,7 @@
       </c>
       <c r="N8" s="15" t="inlineStr">
         <is>
-          <t>Bloque doble con: fuentes de CRM A21–A27 (Claude busca y verifica, Víctor revisa)</t>
+          <t>Bloque doble con: fuentes de CRM A21–A27 (Claude busca y verifica, Víctor revisa) · Adelantada al 19-oct: Cap. I parte 2 v0.1 (justificación, objetivos, metas, alcance); Víctor revisa</t>
         </is>
       </c>
     </row>
@@ -12726,7 +12723,7 @@
       <c r="J10" s="22" t="n"/>
       <c r="K10" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="L10" s="15">
@@ -12740,7 +12737,7 @@
       </c>
       <c r="N10" s="15" t="inlineStr">
         <is>
-          <t>Bloque doble con: censo y métodos A40–A41 (biblioteca UPS: Hernández-Sampieri y Mendoza, 2018)</t>
+          <t>Bloque doble con: censo y métodos A40–A41 (biblioteca UPS: Hernández-Sampieri y Mendoza, 2018) · Adelantada al 19-oct: Cap. II v0.1 con lo verificado (7 fuentes nuevas). Falta CRM móvil (A21–A25) y clásicos de KM</t>
         </is>
       </c>
     </row>
@@ -12850,7 +12847,7 @@
       <c r="J12" s="22" t="n"/>
       <c r="K12" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="L12" s="15">
@@ -12864,7 +12861,7 @@
       </c>
       <c r="N12" s="15" t="inlineStr">
         <is>
-          <t>Bloque doble con: A44 (Ley de Comercio Electrónico) y A30 (blockchain)</t>
+          <t>Bloque doble con: A44 (Ley de Comercio Electrónico) y A30 (blockchain) · Adelantada al 19-oct: va en el mismo Cap. II v0.1 (RAG, normativa). Faltan Lewis 2020, Kleppmann, SHA-256, A44</t>
         </is>
       </c>
     </row>
@@ -12967,10 +12964,12 @@
       <c r="I14" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="J14" s="22" t="n"/>
+      <c r="J14" s="22" t="n">
+        <v>46314</v>
+      </c>
       <c r="K14" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L14" s="15">
@@ -12982,7 +12981,11 @@
           <t>S2-02 (#14)</t>
         </is>
       </c>
-      <c r="N14" s="15" t="inlineStr"/>
+      <c r="N14" s="15" t="inlineStr">
+        <is>
+          <t>19-oct: 4 fichas nuevas de IA (rodriguez_2025, chatterjee_2023a, bohm_2026, hernandezvega_2026) + 10 de CTX-IA ya verificadas</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
@@ -13028,7 +13031,7 @@
       <c r="J15" s="22" t="n"/>
       <c r="K15" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="L15" s="15">
@@ -13040,7 +13043,11 @@
           <t>S2-07 (#58)</t>
         </is>
       </c>
-      <c r="N15" s="15" t="inlineStr"/>
+      <c r="N15" s="15" t="inlineStr">
+        <is>
+          <t>Adelantada al 19-oct: lienzo v0.1 (propuesta de valor para Torvesa + TEAMSLASH como anexo, D7); Víctor revisa</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
@@ -13144,7 +13151,7 @@
       <c r="J17" s="22" t="n"/>
       <c r="K17" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="L17" s="15">
@@ -13156,7 +13163,11 @@
           <t>S2-03 (#15)</t>
         </is>
       </c>
-      <c r="N17" s="15" t="inlineStr"/>
+      <c r="N17" s="15" t="inlineStr">
+        <is>
+          <t>Adelantada al 19-oct: Cap. III completo v0.1 (partes 1 y 2); Víctor revisa</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
@@ -13202,7 +13213,7 @@
       <c r="J18" s="22" t="n"/>
       <c r="K18" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="L18" s="15">
@@ -13214,7 +13225,11 @@
           <t>S2-01 (#13)</t>
         </is>
       </c>
-      <c r="N18" s="15" t="inlineStr"/>
+      <c r="N18" s="15" t="inlineStr">
+        <is>
+          <t>Adelantada al 19-oct: 06_Capitulos/2026-10-19_Resumen_Cap1.md; Víctor lo revisa y lo envía</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
@@ -13376,7 +13391,7 @@
       <c r="J21" s="22" t="n"/>
       <c r="K21" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="L21" s="15">
@@ -13388,7 +13403,11 @@
           <t>S2-03 (#15)</t>
         </is>
       </c>
-      <c r="N21" s="15" t="inlineStr"/>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>Adelantada al 19-oct: va en el mismo Cap. III v0.1; Víctor revisa</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">

</xml_diff>

<commit_message>
v0.1 aprobadas por Víctor y v0.2 de los caps. I, II y III y del lienzo (DEC-16, DEC-17); norma SHA-256 y 2 fuentes nuevas verificadas (40); búsqueda documentada de A28/A29; matriz v0.3; NotebookLM con 29 fuentes y su guía (#13 #14 #15 #58) [IA: Claude]
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/11_Planificacion/Cronograma_Tesis.xlsx
+++ b/11_Planificacion/Cronograma_Tesis.xlsx
@@ -45,11 +45,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="dd-mmm"/>
     <numFmt numFmtId="165" formatCode="dddd"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="dd-mmm-yy"/>
+    <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -156,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -202,6 +203,9 @@
     </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -12472,10 +12476,12 @@
       <c r="I6" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="J6" s="22" t="n"/>
+      <c r="J6" s="27" t="n">
+        <v>46315</v>
+      </c>
       <c r="K6" s="15" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L6" s="15">
@@ -12489,7 +12495,7 @@
       </c>
       <c r="N6" s="15" t="inlineStr">
         <is>
-          <t>Bloque doble con: bajar a mano los PDF de la matriz (Oldroyd, Pollitt, Galan, Nyqvist, Lewis y Sauro, Auernhammer) → Claude los verifica · 19-oct: Cap. I parte 1 v0.1 hecha por Claude (control de cambios); Víctor revisa. PDF a mano: esta noche</t>
+          <t>Bloque doble con: bajar a mano los PDF de la matriz (Oldroyd, Pollitt, Galan, Nyqvist, Lewis y Sauro, Auernhammer) → Claude los verifica · 19-oct: Cap. I parte 1 v0.1 hecha por Claude (control de cambios); Víctor revisa. PDF a mano: esta noche · 20-oct: Víctor aprobó la v0.1; v0.2 en 06_Capitulos/2026-10-20_Cap1_Introduccion_p1_v0.2.docx</t>
         </is>
       </c>
     </row>
@@ -12596,10 +12602,12 @@
       <c r="I8" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="J8" s="22" t="n"/>
+      <c r="J8" s="27" t="n">
+        <v>46315</v>
+      </c>
       <c r="K8" s="15" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L8" s="15">
@@ -12613,7 +12621,7 @@
       </c>
       <c r="N8" s="15" t="inlineStr">
         <is>
-          <t>Bloque doble con: fuentes de CRM A21–A27 (Claude busca y verifica, Víctor revisa) · Adelantada al 19-oct: Cap. I parte 2 v0.1 (justificación, objetivos, metas, alcance); Víctor revisa</t>
+          <t>Bloque doble con: fuentes de CRM A21–A27 (Claude busca y verifica, Víctor revisa) · Adelantada al 19-oct: Cap. I parte 2 v0.1 (justificación, objetivos, metas, alcance); Víctor revisa · 20-oct: Víctor aprobó la v0.1; v0.2 con vacíos A28/A29 documentados (2026-10-20_Cap1_Introduccion_p2_v0.2.docx)</t>
         </is>
       </c>
     </row>
@@ -12720,10 +12728,12 @@
       <c r="I10" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="J10" s="22" t="n"/>
+      <c r="J10" s="27" t="n">
+        <v>46315</v>
+      </c>
       <c r="K10" s="15" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L10" s="15">
@@ -12737,7 +12747,7 @@
       </c>
       <c r="N10" s="15" t="inlineStr">
         <is>
-          <t>Bloque doble con: censo y métodos A40–A41 (biblioteca UPS: Hernández-Sampieri y Mendoza, 2018) · Adelantada al 19-oct: Cap. II v0.1 con lo verificado (7 fuentes nuevas). Falta CRM móvil (A21–A25) y clásicos de KM</t>
+          <t>Bloque doble con: censo y métodos A40–A41 (biblioteca UPS: Hernández-Sampieri y Mendoza, 2018) · Adelantada al 19-oct: Cap. II v0.1 con lo verificado (7 fuentes nuevas). Falta CRM móvil (A21–A25) y clásicos de KM · 20-oct: Víctor aprobó la v0.1; v0.2 con TEAMSLASH como antecedente propio (DEC-17)</t>
         </is>
       </c>
     </row>
@@ -12844,10 +12854,12 @@
       <c r="I12" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="J12" s="22" t="n"/>
+      <c r="J12" s="27" t="n">
+        <v>46315</v>
+      </c>
       <c r="K12" s="15" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L12" s="15">
@@ -12861,7 +12873,7 @@
       </c>
       <c r="N12" s="15" t="inlineStr">
         <is>
-          <t>Bloque doble con: A44 (Ley de Comercio Electrónico) y A30 (blockchain) · Adelantada al 19-oct: va en el mismo Cap. II v0.1 (RAG, normativa). Faltan Lewis 2020, Kleppmann, SHA-256, A44</t>
+          <t>Bloque doble con: A44 (Ley de Comercio Electrónico) y A30 (blockchain) · Adelantada al 19-oct: va en el mismo Cap. II v0.1 (RAG, normativa). Faltan Lewis 2020, Kleppmann, SHA-256, A44 · 20-oct: v0.2 con norma SHA-256 (NIST 2015) y vacíos reformulados (2026-10-20_Cap2_Marco_Teorico_v0.2.docx)</t>
         </is>
       </c>
     </row>
@@ -13028,10 +13040,12 @@
       <c r="I15" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="J15" s="22" t="n"/>
+      <c r="J15" s="27" t="n">
+        <v>46315</v>
+      </c>
       <c r="K15" s="15" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L15" s="15">
@@ -13045,7 +13059,7 @@
       </c>
       <c r="N15" s="15" t="inlineStr">
         <is>
-          <t>Adelantada al 19-oct: lienzo v0.1 (propuesta de valor para Torvesa + TEAMSLASH como anexo, D7); Víctor revisa</t>
+          <t>Adelantada al 19-oct: lienzo v0.1 (propuesta de valor para Torvesa + TEAMSLASH como anexo, D7); Víctor revisa · 20-oct: lienzo v0.2 con DEC-16 (bóveda en Estándar, IA solo en Premium)</t>
         </is>
       </c>
     </row>
@@ -13148,10 +13162,12 @@
       <c r="I17" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="J17" s="22" t="n"/>
+      <c r="J17" s="27" t="n">
+        <v>46315</v>
+      </c>
       <c r="K17" s="15" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L17" s="15">
@@ -13165,7 +13181,7 @@
       </c>
       <c r="N17" s="15" t="inlineStr">
         <is>
-          <t>Adelantada al 19-oct: Cap. III completo v0.1 (partes 1 y 2); Víctor revisa</t>
+          <t>Adelantada al 19-oct: Cap. III completo v0.1 (partes 1 y 2); Víctor revisa · 20-oct: Víctor aprobó la v0.1; v0.2 (2026-10-20_Cap3_Metodologia_v0.2.docx)</t>
         </is>
       </c>
     </row>
@@ -13388,10 +13404,12 @@
       <c r="I21" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="J21" s="22" t="n"/>
+      <c r="J21" s="27" t="n">
+        <v>46315</v>
+      </c>
       <c r="K21" s="15" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L21" s="15">
@@ -13405,7 +13423,7 @@
       </c>
       <c r="N21" s="15" t="inlineStr">
         <is>
-          <t>Adelantada al 19-oct: va en el mismo Cap. III v0.1; Víctor revisa</t>
+          <t>Adelantada al 19-oct: va en el mismo Cap. III v0.1; Víctor revisa · 20-oct: va en el mismo Cap. III v0.2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revisión 1 y puesta al día: caps. I–III v0.3, hoja de puntos, presentación y guion para la tutora; elicitación y análisis de requerimientos v0.1 (ISO/IEC/IEEE 29148 + SWEBOK, 23 requerimientos) y planteamiento del problema; auditoría de Diego, cronograma reprogramado, IA_DIEGO v0.2 y bitácora 22–27 oct [IA: Claude]
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/11_Planificacion/Cronograma_Tesis.xlsx
+++ b/11_Planificacion/Cronograma_Tesis.xlsx
@@ -27,8 +27,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'S1'!$A$5:$N$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'S2'!$A$5:$N$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'S3'!$A$5:$N$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'S4'!$A$5:$N$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'S3'!$A$5:$N$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'S4'!$A$5:$N$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'S5'!$A$5:$N$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'S6'!$A$5:$N$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'S7'!$A$5:$N$19</definedName>
@@ -45,12 +45,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="dd-mmm"/>
     <numFmt numFmtId="165" formatCode="dddd"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="dd-mmm-yy"/>
     <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="169" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -6029,6 +6030,7 @@
       <c r="M2" s="2" t="n"/>
       <c r="N2" s="2" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -6181,11 +6183,11 @@
         </is>
       </c>
       <c r="C7" s="7">
-        <f>COUNTA('S3'!D6:D19)-COUNTIF('S3'!K6:K19,"Cancelado")</f>
+        <f>COUNTA('S3'!D6:D24)-COUNTIF('S3'!K6:K24,"Cancelado")</f>
         <v/>
       </c>
       <c r="D7" s="7">
-        <f>COUNTIF('S3'!K6:K19,"Hecho")</f>
+        <f>COUNTIF('S3'!K6:K24,"Hecho")</f>
         <v/>
       </c>
       <c r="E7" s="8">
@@ -6193,23 +6195,23 @@
         <v/>
       </c>
       <c r="F7" s="8">
-        <f>IFERROR((COUNTIFS('S3'!E6:E19,"Víctor",'S3'!K6:K19,"Hecho")+COUNTIFS('S3'!E6:E19,"Ambos",'S3'!K6:K19,"Hecho"))/(COUNTIF('S3'!E6:E19,"Víctor")+COUNTIF('S3'!E6:E19,"Ambos")),0)</f>
+        <f>IFERROR((COUNTIFS('S3'!E6:E24,"Víctor",'S3'!K6:K24,"Hecho")+COUNTIFS('S3'!E6:E24,"Ambos",'S3'!K6:K24,"Hecho"))/(COUNTIF('S3'!E6:E24,"Víctor")+COUNTIF('S3'!E6:E24,"Ambos")),0)</f>
         <v/>
       </c>
       <c r="G7" s="8">
-        <f>IFERROR((COUNTIFS('S3'!E6:E19,"Diego",'S3'!K6:K19,"Hecho")+COUNTIFS('S3'!E6:E19,"Ambos",'S3'!K6:K19,"Hecho"))/(COUNTIF('S3'!E6:E19,"Diego")+COUNTIF('S3'!E6:E19,"Ambos")),0)</f>
+        <f>IFERROR((COUNTIFS('S3'!E6:E24,"Diego",'S3'!K6:K24,"Hecho")+COUNTIFS('S3'!E6:E24,"Ambos",'S3'!K6:K24,"Hecho"))/(COUNTIF('S3'!E6:E24,"Diego")+COUNTIF('S3'!E6:E24,"Ambos")),0)</f>
         <v/>
       </c>
       <c r="H7" s="7">
-        <f>SUMIF('S3'!E6:E19,"Víctor",'S3'!I6:I19)+SUMIF('S3'!E6:E19,"Ambos",'S3'!I6:I19)</f>
+        <f>SUMIF('S3'!E6:E24,"Víctor",'S3'!I6:I24)+SUMIF('S3'!E6:E24,"Ambos",'S3'!I6:I24)</f>
         <v/>
       </c>
       <c r="I7" s="7">
-        <f>SUMIF('S3'!E6:E19,"Diego",'S3'!I6:I19)+SUMIF('S3'!E6:E19,"Ambos",'S3'!I6:I19)</f>
+        <f>SUMIF('S3'!E6:E24,"Diego",'S3'!I6:I24)+SUMIF('S3'!E6:E24,"Ambos",'S3'!I6:I24)</f>
         <v/>
       </c>
       <c r="J7" s="7">
-        <f>COUNTIF('S3'!L6:L19,"&gt;0")</f>
+        <f>COUNTIF('S3'!L6:L24,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -6225,11 +6227,11 @@
         </is>
       </c>
       <c r="C8" s="7">
-        <f>COUNTA('S4'!D6:D20)-COUNTIF('S4'!K6:K20,"Cancelado")</f>
+        <f>COUNTA('S4'!D6:D22)-COUNTIF('S4'!K6:K22,"Cancelado")</f>
         <v/>
       </c>
       <c r="D8" s="7">
-        <f>COUNTIF('S4'!K6:K20,"Hecho")</f>
+        <f>COUNTIF('S4'!K6:K22,"Hecho")</f>
         <v/>
       </c>
       <c r="E8" s="8">
@@ -6237,23 +6239,23 @@
         <v/>
       </c>
       <c r="F8" s="8">
-        <f>IFERROR((COUNTIFS('S4'!E6:E20,"Víctor",'S4'!K6:K20,"Hecho")+COUNTIFS('S4'!E6:E20,"Ambos",'S4'!K6:K20,"Hecho"))/(COUNTIF('S4'!E6:E20,"Víctor")+COUNTIF('S4'!E6:E20,"Ambos")),0)</f>
+        <f>IFERROR((COUNTIFS('S4'!E6:E22,"Víctor",'S4'!K6:K22,"Hecho")+COUNTIFS('S4'!E6:E22,"Ambos",'S4'!K6:K22,"Hecho"))/(COUNTIF('S4'!E6:E22,"Víctor")+COUNTIF('S4'!E6:E22,"Ambos")),0)</f>
         <v/>
       </c>
       <c r="G8" s="8">
-        <f>IFERROR((COUNTIFS('S4'!E6:E20,"Diego",'S4'!K6:K20,"Hecho")+COUNTIFS('S4'!E6:E20,"Ambos",'S4'!K6:K20,"Hecho"))/(COUNTIF('S4'!E6:E20,"Diego")+COUNTIF('S4'!E6:E20,"Ambos")),0)</f>
+        <f>IFERROR((COUNTIFS('S4'!E6:E22,"Diego",'S4'!K6:K22,"Hecho")+COUNTIFS('S4'!E6:E22,"Ambos",'S4'!K6:K22,"Hecho"))/(COUNTIF('S4'!E6:E22,"Diego")+COUNTIF('S4'!E6:E22,"Ambos")),0)</f>
         <v/>
       </c>
       <c r="H8" s="7">
-        <f>SUMIF('S4'!E6:E20,"Víctor",'S4'!I6:I20)+SUMIF('S4'!E6:E20,"Ambos",'S4'!I6:I20)</f>
+        <f>SUMIF('S4'!E6:E22,"Víctor",'S4'!I6:I22)+SUMIF('S4'!E6:E22,"Ambos",'S4'!I6:I22)</f>
         <v/>
       </c>
       <c r="I8" s="7">
-        <f>SUMIF('S4'!E6:E20,"Diego",'S4'!I6:I20)+SUMIF('S4'!E6:E20,"Ambos",'S4'!I6:I20)</f>
+        <f>SUMIF('S4'!E6:E22,"Diego",'S4'!I6:I22)+SUMIF('S4'!E6:E22,"Ambos",'S4'!I6:I22)</f>
         <v/>
       </c>
       <c r="J8" s="7">
-        <f>COUNTIF('S4'!L6:L20,"&gt;0")</f>
+        <f>COUNTIF('S4'!L6:L22,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -7085,10 +7087,12 @@
       <c r="I9" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="J9" s="22" t="n"/>
+      <c r="J9" s="22" t="n">
+        <v>46314</v>
+      </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L9" s="15">
@@ -7102,7 +7106,7 @@
       </c>
       <c r="N9" s="15" t="inlineStr">
         <is>
-          <t>Diego acepta la invitación el 18-oct (vencía ese día)</t>
+          <t>Diego acepta la invitación el 18-oct (vencía ese día) · 19-oct: repo clonado y commit de prueba (00_Inbox/hola_diego.md)</t>
         </is>
       </c>
     </row>
@@ -7147,10 +7151,12 @@
       <c r="I10" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="J10" s="22" t="n"/>
+      <c r="J10" s="22" t="n">
+        <v>46314</v>
+      </c>
       <c r="K10" s="15" t="inlineStr">
         <is>
-          <t>Movido</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L10" s="15">
@@ -7164,7 +7170,7 @@
       </c>
       <c r="N10" s="15" t="inlineStr">
         <is>
-          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md)</t>
+          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md) · 19-oct: RAG funcionando en la PC de Diego (586 notas indexadas)</t>
         </is>
       </c>
     </row>
@@ -7335,10 +7341,12 @@
       <c r="I13" s="24" t="n">
         <v>1.5</v>
       </c>
-      <c r="J13" s="22" t="n"/>
+      <c r="J13" s="22" t="n">
+        <v>46316</v>
+      </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>Movido</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L13" s="15">
@@ -7352,7 +7360,7 @@
       </c>
       <c r="N13" s="15" t="inlineStr">
         <is>
-          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md)</t>
+          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md) · 21-oct: 7 fichas verificadas de gestión del conocimiento (D01)</t>
         </is>
       </c>
     </row>
@@ -7397,10 +7405,12 @@
       <c r="I14" s="24" t="n">
         <v>0.5</v>
       </c>
-      <c r="J14" s="22" t="n"/>
+      <c r="J14" s="22" t="n">
+        <v>46314</v>
+      </c>
       <c r="K14" s="15" t="inlineStr">
         <is>
-          <t>Movido</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L14" s="15">
@@ -7414,7 +7424,7 @@
       </c>
       <c r="N14" s="15" t="inlineStr">
         <is>
-          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md)</t>
+          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md) · 19-oct: leído; 5 dudas en 00_Inbox/2026-10-19_reporte_Diego.md</t>
         </is>
       </c>
     </row>
@@ -7649,10 +7659,12 @@
       <c r="I18" s="24" t="n">
         <v>1.5</v>
       </c>
-      <c r="J18" s="22" t="n"/>
+      <c r="J18" s="22" t="n">
+        <v>46316</v>
+      </c>
       <c r="K18" s="15" t="inlineStr">
         <is>
-          <t>Movido</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L18" s="15">
@@ -7666,7 +7678,7 @@
       </c>
       <c r="N18" s="15" t="inlineStr">
         <is>
-          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md)</t>
+          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md) · 21-oct: 6 fichas verificadas de RAG (D02); A37 cubierta</t>
         </is>
       </c>
     </row>
@@ -7711,10 +7723,12 @@
       <c r="I19" s="24" t="n">
         <v>0.5</v>
       </c>
-      <c r="J19" s="22" t="n"/>
+      <c r="J19" s="22" t="n">
+        <v>46320</v>
+      </c>
       <c r="K19" s="15" t="inlineStr">
         <is>
-          <t>Movido</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L19" s="15">
@@ -7728,7 +7742,7 @@
       </c>
       <c r="N19" s="15" t="inlineStr">
         <is>
-          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md)</t>
+          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md) · 25-oct: 02_Fuentes/Tecnologia_IA/2026-10-25_Resumen_Bovedas_RAG.md</t>
         </is>
       </c>
     </row>
@@ -7852,7 +7866,7 @@
       </c>
       <c r="N21" s="15" t="inlineStr">
         <is>
-          <t>Movido: se aplica cuando Torvesa autorice (Diego consigue la información y los permisos)</t>
+          <t>Movido: se aplica cuando Torvesa autorice (Diego consigue la información y los permisos) · 27-oct: bloqueada, Torvesa aún no autoriza el campo; copia en S4-T16 (reprogramada 27-oct)</t>
         </is>
       </c>
     </row>
@@ -7976,7 +7990,7 @@
       </c>
       <c r="N23" s="15" t="inlineStr">
         <is>
-          <t>Movido: se aplica cuando Torvesa autorice (Diego consigue la información y los permisos)</t>
+          <t>Movido: se aplica cuando Torvesa autorice (Diego consigue la información y los permisos) · 27-oct: bloqueada, Torvesa aún no autoriza el campo; copia en S4-T16 (reprogramada 27-oct)</t>
         </is>
       </c>
     </row>
@@ -8211,10 +8225,12 @@
       <c r="I27" s="24" t="n">
         <v>1.5</v>
       </c>
-      <c r="J27" s="22" t="n"/>
+      <c r="J27" s="22" t="n">
+        <v>46320</v>
+      </c>
       <c r="K27" s="15" t="inlineStr">
         <is>
-          <t>Movido</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L27" s="15">
@@ -8228,7 +8244,7 @@
       </c>
       <c r="N27" s="15" t="inlineStr">
         <is>
-          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md)</t>
+          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md) · 25-oct: 6 fichas verificadas de BPMN y procesos, incluida la especificación OMG</t>
         </is>
       </c>
     </row>
@@ -8273,10 +8289,12 @@
       <c r="I28" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="J28" s="22" t="n"/>
+      <c r="J28" s="22" t="n">
+        <v>46320</v>
+      </c>
       <c r="K28" s="15" t="inlineStr">
         <is>
-          <t>Movido</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L28" s="15">
@@ -8290,7 +8308,7 @@
       </c>
       <c r="N28" s="15" t="inlineStr">
         <is>
-          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md)</t>
+          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md) · 25-oct: fichas de precios de CRM, mensajería, bóveda y LLM (bloques G y H)</t>
         </is>
       </c>
     </row>
@@ -8352,7 +8370,7 @@
       </c>
       <c r="N29" s="15" t="inlineStr">
         <is>
-          <t>Movido: se aplica cuando Torvesa autorice (Diego consigue la información y los permisos). Al día siguiente del campo</t>
+          <t>Movido: se aplica cuando Torvesa autorice (Diego consigue la información y los permisos). Al día siguiente del campo · 27-oct: bloqueada, sin datos de campo; se hace al día siguiente del campo (S4-T16)</t>
         </is>
       </c>
     </row>
@@ -8461,10 +8479,12 @@
       <c r="I31" s="24" t="n">
         <v>0.5</v>
       </c>
-      <c r="J31" s="22" t="n"/>
+      <c r="J31" s="22" t="n">
+        <v>46320</v>
+      </c>
       <c r="K31" s="15" t="inlineStr">
         <is>
-          <t>Movido</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L31" s="15">
@@ -8478,7 +8498,7 @@
       </c>
       <c r="N31" s="15" t="inlineStr">
         <is>
-          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md)</t>
+          <t>Movido a la semana 19–24 oct (bloques dobles de Diego en IA_DIEGO.md) · 25-oct: 02_Fuentes/Casos_Estudio/2026-10-25_Resumen_CRM_Flujos.md</t>
         </is>
       </c>
     </row>
@@ -8630,6 +8650,7 @@
       <c r="M2" s="2" t="n"/>
       <c r="N2" s="2" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -8680,19 +8701,19 @@
         <v/>
       </c>
       <c r="D5" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A5,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A5,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A5,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A5,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A5,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A5,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A5,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A5,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E5" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A5,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A5,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A5,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A5,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A5,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A5,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A5,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A5,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F5" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A5,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A5,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A5,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A5,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A5,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A5,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A5,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A5,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G5" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A5,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A5,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A5,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A5,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A5,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A5,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A5,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A5,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A5,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A5,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A5,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A5,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A5,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A5,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A5,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A5,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A5,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A5,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A5,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -8709,19 +8730,19 @@
         <v/>
       </c>
       <c r="D6" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A6,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A6,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A6,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A6,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A6,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A6,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A6,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A6,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E6" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A6,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A6,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A6,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A6,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A6,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A6,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A6,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A6,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F6" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A6,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A6,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A6,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A6,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A6,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A6,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A6,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A6,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G6" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A6,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A6,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A6,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A6,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A6,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A6,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A6,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A6,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A6,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A6,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A6,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A6,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A6,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A6,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A6,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A6,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A6,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A6,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A6,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -8738,19 +8759,19 @@
         <v/>
       </c>
       <c r="D7" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A7,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A7,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A7,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A7,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A7,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A7,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A7,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A7,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E7" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A7,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A7,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A7,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A7,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A7,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A7,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A7,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A7,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F7" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A7,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A7,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A7,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A7,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A7,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A7,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A7,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A7,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G7" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A7,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A7,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A7,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A7,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A7,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A7,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A7,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A7,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A7,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A7,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A7,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A7,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A7,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A7,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A7,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A7,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A7,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A7,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A7,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -8767,19 +8788,19 @@
         <v/>
       </c>
       <c r="D8" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A8,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A8,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A8,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A8,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A8,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A8,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A8,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A8,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E8" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A8,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A8,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A8,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A8,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A8,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A8,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A8,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A8,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F8" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A8,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A8,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A8,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A8,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A8,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A8,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A8,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A8,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G8" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A8,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A8,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A8,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A8,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A8,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A8,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A8,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A8,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A8,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A8,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A8,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A8,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A8,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A8,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A8,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A8,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A8,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A8,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A8,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -8796,19 +8817,19 @@
         <v/>
       </c>
       <c r="D9" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A9,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A9,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A9,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A9,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A9,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A9,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A9,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A9,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E9" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A9,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A9,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A9,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A9,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A9,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A9,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A9,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A9,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F9" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A9,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A9,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A9,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A9,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A9,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A9,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A9,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A9,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G9" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A9,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A9,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A9,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A9,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A9,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A9,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A9,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A9,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A9,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A9,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A9,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A9,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A9,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A9,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A9,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A9,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A9,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A9,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A9,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -8825,19 +8846,19 @@
         <v/>
       </c>
       <c r="D10" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A10,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A10,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A10,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A10,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A10,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A10,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A10,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A10,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E10" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A10,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A10,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A10,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A10,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A10,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A10,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A10,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A10,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F10" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A10,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A10,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A10,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A10,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A10,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A10,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A10,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A10,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G10" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A10,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A10,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A10,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A10,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A10,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A10,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A10,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A10,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A10,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A10,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A10,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A10,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A10,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A10,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A10,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A10,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A10,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A10,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A10,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -8854,19 +8875,19 @@
         <v/>
       </c>
       <c r="D11" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A11,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A11,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A11,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A11,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A11,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A11,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A11,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A11,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E11" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A11,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A11,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A11,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A11,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A11,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A11,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A11,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A11,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F11" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A11,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A11,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A11,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A11,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A11,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A11,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A11,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A11,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G11" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A11,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A11,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A11,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A11,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A11,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A11,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A11,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A11,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A11,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A11,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A11,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A11,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A11,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A11,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A11,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A11,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A11,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A11,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A11,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -8883,19 +8904,19 @@
         <v/>
       </c>
       <c r="D12" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A12,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A12,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A12,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A12,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A12,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A12,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A12,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A12,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E12" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A12,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A12,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A12,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A12,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A12,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A12,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A12,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A12,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F12" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A12,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A12,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A12,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A12,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A12,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A12,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A12,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A12,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G12" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A12,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A12,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A12,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A12,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A12,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A12,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A12,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A12,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A12,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A12,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A12,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A12,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A12,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A12,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A12,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A12,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A12,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A12,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A12,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -8912,19 +8933,19 @@
         <v/>
       </c>
       <c r="D13" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A13,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A13,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A13,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A13,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A13,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A13,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A13,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A13,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E13" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A13,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A13,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A13,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A13,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A13,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A13,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A13,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A13,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F13" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A13,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A13,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A13,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A13,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A13,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A13,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A13,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A13,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G13" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A13,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A13,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A13,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A13,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A13,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A13,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A13,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A13,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A13,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A13,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A13,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A13,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A13,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A13,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A13,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A13,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A13,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A13,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A13,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -8941,19 +8962,19 @@
         <v/>
       </c>
       <c r="D14" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A14,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A14,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A14,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A14,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A14,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A14,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A14,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A14,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E14" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A14,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A14,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A14,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A14,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A14,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A14,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A14,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A14,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F14" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A14,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A14,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A14,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A14,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A14,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A14,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A14,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A14,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G14" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A14,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A14,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A14,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A14,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A14,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A14,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A14,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A14,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A14,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A14,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A14,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A14,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A14,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A14,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A14,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A14,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A14,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A14,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A14,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -8970,19 +8991,19 @@
         <v/>
       </c>
       <c r="D15" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A15,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A15,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A15,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A15,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A15,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A15,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A15,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A15,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E15" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A15,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A15,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A15,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A15,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A15,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A15,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A15,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A15,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F15" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A15,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A15,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A15,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A15,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A15,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A15,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A15,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A15,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A15,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A15,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A15,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A15,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A15,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A15,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A15,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A15,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A15,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A15,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A15,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A15,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A15,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A15,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A15,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A15,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A15,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A15,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A15,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -8999,19 +9020,19 @@
         <v/>
       </c>
       <c r="D16" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A16,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A16,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A16,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A16,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A16,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A16,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A16,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A16,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E16" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A16,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A16,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A16,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A16,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A16,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A16,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A16,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A16,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F16" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A16,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A16,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A16,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A16,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A16,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A16,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A16,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A16,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G16" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A16,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A16,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A16,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A16,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A16,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A16,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A16,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A16,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A16,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A16,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A16,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A16,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A16,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A16,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A16,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A16,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A16,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A16,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A16,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9028,19 +9049,19 @@
         <v/>
       </c>
       <c r="D17" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A17,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A17,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A17,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A17,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A17,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A17,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A17,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A17,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E17" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A17,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A17,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A17,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A17,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A17,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A17,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A17,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A17,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F17" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A17,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A17,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A17,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A17,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A17,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A17,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A17,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A17,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G17" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A17,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A17,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A17,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A17,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A17,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A17,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A17,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A17,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A17,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A17,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A17,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A17,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A17,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A17,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A17,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A17,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A17,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A17,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A17,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9057,19 +9078,19 @@
         <v/>
       </c>
       <c r="D18" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A18,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A18,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A18,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A18,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A18,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A18,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A18,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A18,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E18" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A18,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A18,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A18,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A18,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A18,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A18,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A18,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A18,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F18" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A18,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A18,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A18,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A18,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A18,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A18,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A18,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A18,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G18" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A18,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A18,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A18,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A18,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A18,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A18,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A18,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A18,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A18,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A18,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A18,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A18,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A18,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A18,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A18,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A18,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A18,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A18,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A18,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9086,19 +9107,19 @@
         <v/>
       </c>
       <c r="D19" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A19,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A19,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A19,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A19,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A19,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A19,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A19,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A19,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E19" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A19,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A19,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A19,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A19,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A19,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A19,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A19,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A19,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F19" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A19,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A19,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A19,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A19,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A19,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A19,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A19,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A19,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G19" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A19,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A19,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A19,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A19,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A19,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A19,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A19,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A19,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A19,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A19,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A19,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A19,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A19,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A19,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A19,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A19,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A19,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A19,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A19,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9115,19 +9136,19 @@
         <v/>
       </c>
       <c r="D20" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A20,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A20,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A20,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A20,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A20,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A20,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A20,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A20,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E20" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A20,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A20,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A20,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A20,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A20,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A20,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A20,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A20,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F20" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A20,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A20,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A20,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A20,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A20,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A20,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A20,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A20,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G20" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A20,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A20,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A20,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A20,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A20,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A20,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A20,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A20,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A20,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A20,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A20,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A20,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A20,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A20,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A20,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A20,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A20,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A20,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A20,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9144,19 +9165,19 @@
         <v/>
       </c>
       <c r="D21" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A21,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A21,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A21,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A21,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A21,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A21,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A21,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A21,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E21" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A21,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A21,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A21,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A21,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A21,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A21,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A21,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A21,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F21" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A21,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A21,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A21,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A21,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A21,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A21,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A21,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A21,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G21" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A21,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A21,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A21,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A21,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A21,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A21,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A21,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A21,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A21,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A21,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A21,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A21,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A21,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A21,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A21,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A21,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A21,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A21,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A21,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9173,19 +9194,19 @@
         <v/>
       </c>
       <c r="D22" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A22,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A22,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A22,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A22,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A22,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A22,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A22,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A22,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E22" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A22,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A22,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A22,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A22,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A22,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A22,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A22,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A22,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F22" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A22,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A22,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A22,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A22,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A22,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A22,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A22,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A22,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G22" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A22,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A22,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A22,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A22,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A22,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A22,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A22,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A22,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A22,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A22,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A22,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A22,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A22,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A22,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A22,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A22,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A22,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A22,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A22,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9202,19 +9223,19 @@
         <v/>
       </c>
       <c r="D23" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A23,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A23,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A23,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A23,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A23,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A23,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A23,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A23,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E23" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A23,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A23,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A23,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A23,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A23,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A23,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A23,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A23,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F23" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A23,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A23,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A23,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A23,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A23,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A23,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A23,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A23,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G23" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A23,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A23,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A23,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A23,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A23,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A23,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A23,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A23,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A23,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A23,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A23,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A23,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A23,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A23,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A23,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A23,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A23,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A23,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A23,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9231,19 +9252,19 @@
         <v/>
       </c>
       <c r="D24" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A24,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A24,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A24,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A24,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A24,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A24,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A24,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A24,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E24" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A24,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A24,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A24,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A24,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A24,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A24,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A24,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A24,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F24" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A24,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A24,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A24,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A24,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A24,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A24,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A24,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A24,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G24" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A24,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A24,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A24,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A24,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A24,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A24,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A24,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A24,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A24,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A24,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A24,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A24,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A24,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A24,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A24,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A24,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A24,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A24,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A24,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9260,19 +9281,19 @@
         <v/>
       </c>
       <c r="D25" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A25,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A25,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A25,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A25,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A25,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A25,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A25,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A25,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E25" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A25,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A25,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A25,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A25,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A25,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A25,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A25,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A25,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F25" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A25,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A25,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A25,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A25,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A25,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A25,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A25,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A25,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G25" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A25,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A25,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A25,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A25,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A25,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A25,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A25,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A25,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A25,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A25,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A25,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A25,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A25,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A25,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A25,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A25,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A25,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A25,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A25,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9289,19 +9310,19 @@
         <v/>
       </c>
       <c r="D26" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A26,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A26,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A26,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A26,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A26,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A26,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A26,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A26,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E26" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A26,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A26,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A26,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A26,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A26,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A26,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A26,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A26,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F26" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A26,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A26,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A26,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A26,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A26,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A26,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A26,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A26,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G26" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A26,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A26,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A26,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A26,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A26,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A26,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A26,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A26,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A26,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A26,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A26,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A26,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A26,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A26,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A26,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A26,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A26,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A26,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A26,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9318,19 +9339,19 @@
         <v/>
       </c>
       <c r="D27" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A27,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A27,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A27,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A27,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A27,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A27,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A27,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A27,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E27" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A27,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A27,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A27,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A27,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A27,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A27,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A27,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A27,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F27" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A27,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A27,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A27,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A27,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A27,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A27,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A27,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A27,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G27" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A27,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A27,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A27,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A27,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A27,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A27,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A27,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A27,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A27,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A27,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A27,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A27,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A27,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A27,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A27,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A27,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A27,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A27,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A27,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9347,19 +9368,19 @@
         <v/>
       </c>
       <c r="D28" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A28,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A28,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A28,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A28,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A28,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A28,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A28,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A28,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E28" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A28,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A28,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A28,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A28,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A28,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A28,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A28,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A28,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F28" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A28,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A28,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A28,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A28,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A28,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A28,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A28,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A28,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G28" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A28,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A28,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A28,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A28,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A28,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A28,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A28,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A28,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A28,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A28,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A28,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A28,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A28,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A28,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A28,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A28,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A28,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A28,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A28,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9376,19 +9397,19 @@
         <v/>
       </c>
       <c r="D29" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A29,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A29,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A29,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A29,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A29,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A29,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A29,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A29,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E29" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A29,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A29,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A29,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A29,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A29,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A29,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A29,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A29,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F29" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A29,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A29,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A29,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A29,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A29,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A29,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A29,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A29,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G29" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A29,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A29,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A29,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A29,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A29,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A29,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A29,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A29,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A29,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A29,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A29,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A29,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A29,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A29,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A29,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A29,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A29,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A29,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A29,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9405,19 +9426,19 @@
         <v/>
       </c>
       <c r="D30" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A30,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A30,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A30,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A30,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A30,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A30,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A30,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A30,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E30" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A30,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A30,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A30,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A30,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A30,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A30,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A30,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A30,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F30" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A30,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A30,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A30,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A30,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A30,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A30,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A30,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A30,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G30" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A30,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A30,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A30,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A30,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A30,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A30,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A30,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A30,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A30,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A30,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A30,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A30,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A30,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A30,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A30,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A30,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A30,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A30,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A30,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9434,19 +9455,19 @@
         <v/>
       </c>
       <c r="D31" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A31,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A31,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A31,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A31,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A31,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A31,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A31,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A31,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E31" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A31,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A31,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A31,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A31,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A31,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A31,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A31,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A31,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F31" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A31,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A31,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A31,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A31,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A31,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A31,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A31,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A31,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G31" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A31,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A31,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A31,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A31,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A31,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A31,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A31,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A31,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A31,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A31,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A31,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A31,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A31,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A31,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A31,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A31,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A31,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A31,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A31,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9463,19 +9484,19 @@
         <v/>
       </c>
       <c r="D32" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A32,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A32,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A32,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A32,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A32,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A32,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A32,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A32,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E32" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A32,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A32,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A32,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A32,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A32,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A32,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A32,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A32,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F32" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A32,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A32,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A32,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A32,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A32,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A32,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A32,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A32,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G32" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A32,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A32,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A32,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A32,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A32,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A32,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A32,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A32,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A32,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A32,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A32,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A32,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A32,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A32,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A32,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A32,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A32,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A32,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A32,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9492,19 +9513,19 @@
         <v/>
       </c>
       <c r="D33" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A33,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A33,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A33,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A33,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A33,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A33,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A33,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A33,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E33" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A33,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A33,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A33,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A33,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A33,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A33,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A33,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A33,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F33" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A33,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A33,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A33,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A33,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A33,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A33,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A33,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A33,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G33" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A33,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A33,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A33,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A33,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A33,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A33,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A33,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A33,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A33,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A33,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A33,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A33,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A33,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A33,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A33,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A33,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A33,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A33,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A33,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9521,19 +9542,19 @@
         <v/>
       </c>
       <c r="D34" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A34,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A34,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A34,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A34,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A34,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A34,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A34,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A34,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E34" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A34,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A34,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A34,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A34,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A34,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A34,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A34,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A34,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F34" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A34,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A34,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A34,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A34,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A34,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A34,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A34,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A34,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G34" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A34,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A34,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A34,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A34,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A34,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A34,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A34,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A34,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A34,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A34,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A34,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A34,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A34,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A34,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A34,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A34,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A34,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A34,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A34,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9550,19 +9571,19 @@
         <v/>
       </c>
       <c r="D35" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A35,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A35,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A35,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A35,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A35,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A35,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A35,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A35,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E35" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A35,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A35,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A35,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A35,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A35,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A35,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A35,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A35,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F35" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A35,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A35,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A35,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A35,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A35,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A35,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A35,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A35,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G35" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A35,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A35,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A35,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A35,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A35,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A35,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A35,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A35,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A35,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A35,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A35,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A35,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A35,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A35,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A35,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A35,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A35,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A35,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A35,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9579,19 +9600,19 @@
         <v/>
       </c>
       <c r="D36" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A36,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A36,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A36,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A36,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A36,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A36,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A36,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A36,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E36" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A36,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A36,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A36,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A36,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A36,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A36,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A36,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A36,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F36" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A36,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A36,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A36,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A36,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A36,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A36,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A36,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A36,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G36" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A36,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A36,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A36,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A36,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A36,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A36,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A36,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A36,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A36,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A36,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A36,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A36,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A36,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A36,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A36,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A36,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A36,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A36,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A36,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9608,19 +9629,19 @@
         <v/>
       </c>
       <c r="D37" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A37,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A37,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A37,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A37,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A37,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A37,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A37,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A37,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E37" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A37,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A37,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A37,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A37,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A37,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A37,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A37,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A37,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F37" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A37,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A37,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A37,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A37,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A37,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A37,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A37,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A37,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G37" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A37,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A37,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A37,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A37,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A37,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A37,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A37,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A37,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A37,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A37,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A37,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A37,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A37,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A37,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A37,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A37,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A37,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A37,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A37,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9637,19 +9658,19 @@
         <v/>
       </c>
       <c r="D38" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A38,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A38,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A38,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A38,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A38,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A38,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A38,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A38,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E38" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A38,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A38,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A38,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A38,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A38,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A38,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A38,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A38,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F38" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A38,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A38,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A38,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A38,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A38,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A38,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A38,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A38,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G38" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A38,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A38,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A38,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A38,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A38,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A38,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A38,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A38,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A38,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A38,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A38,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A38,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A38,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A38,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A38,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A38,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A38,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A38,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A38,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9666,19 +9687,19 @@
         <v/>
       </c>
       <c r="D39" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A39,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A39,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A39,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A39,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A39,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A39,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A39,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A39,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E39" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A39,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A39,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A39,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A39,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A39,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A39,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A39,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A39,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F39" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A39,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A39,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A39,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A39,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A39,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A39,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A39,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A39,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G39" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A39,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A39,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A39,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A39,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A39,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A39,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A39,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A39,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A39,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A39,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A39,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A39,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A39,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A39,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A39,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A39,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A39,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A39,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A39,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9695,19 +9716,19 @@
         <v/>
       </c>
       <c r="D40" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A40,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A40,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A40,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A40,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A40,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A40,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A40,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A40,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E40" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A40,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A40,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A40,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A40,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A40,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A40,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A40,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A40,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F40" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A40,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A40,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A40,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A40,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A40,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A40,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A40,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A40,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G40" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A40,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A40,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A40,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A40,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A40,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A40,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A40,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A40,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A40,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A40,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A40,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A40,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A40,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A40,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A40,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A40,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A40,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A40,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A40,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9724,19 +9745,19 @@
         <v/>
       </c>
       <c r="D41" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A41,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A41,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A41,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A41,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A41,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A41,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A41,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A41,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E41" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A41,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A41,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A41,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A41,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A41,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A41,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A41,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A41,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F41" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A41,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A41,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A41,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A41,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A41,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A41,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A41,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A41,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G41" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A41,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A41,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A41,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A41,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A41,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A41,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A41,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A41,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A41,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A41,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A41,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A41,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A41,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A41,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A41,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A41,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A41,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A41,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A41,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9753,19 +9774,19 @@
         <v/>
       </c>
       <c r="D42" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A42,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A42,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A42,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A42,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A42,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A42,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A42,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A42,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E42" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A42,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A42,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A42,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A42,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A42,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A42,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A42,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A42,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F42" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A42,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A42,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A42,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A42,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A42,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A42,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A42,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A42,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G42" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A42,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A42,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A42,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A42,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A42,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A42,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A42,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A42,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A42,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A42,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A42,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A42,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A42,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A42,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A42,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A42,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A42,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A42,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A42,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9782,19 +9803,19 @@
         <v/>
       </c>
       <c r="D43" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A43,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A43,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A43,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A43,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A43,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A43,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A43,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A43,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E43" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A43,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A43,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A43,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A43,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A43,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A43,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A43,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A43,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F43" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A43,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A43,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A43,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A43,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A43,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A43,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A43,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A43,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G43" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A43,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A43,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A43,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A43,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A43,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A43,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A43,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A43,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A43,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A43,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A43,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A43,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A43,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A43,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A43,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A43,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A43,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A43,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A43,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9811,19 +9832,19 @@
         <v/>
       </c>
       <c r="D44" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A44,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A44,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A44,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A44,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A44,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A44,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A44,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A44,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E44" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A44,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A44,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A44,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A44,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A44,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A44,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A44,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A44,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F44" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A44,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A44,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A44,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A44,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A44,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A44,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A44,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A44,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G44" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A44,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A44,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A44,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A44,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A44,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A44,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A44,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A44,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A44,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A44,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A44,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A44,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A44,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A44,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A44,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A44,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A44,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A44,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A44,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9840,19 +9861,19 @@
         <v/>
       </c>
       <c r="D45" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A45,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A45,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A45,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A45,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A45,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A45,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A45,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A45,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E45" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A45,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A45,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A45,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A45,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A45,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A45,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A45,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A45,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F45" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A45,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A45,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A45,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A45,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A45,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A45,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A45,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A45,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G45" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A45,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A45,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A45,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A45,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A45,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A45,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A45,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A45,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A45,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A45,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A45,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A45,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A45,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A45,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A45,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A45,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A45,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A45,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A45,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9869,19 +9890,19 @@
         <v/>
       </c>
       <c r="D46" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A46,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A46,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A46,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A46,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A46,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A46,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A46,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A46,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E46" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A46,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A46,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A46,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A46,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A46,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A46,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A46,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A46,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F46" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A46,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A46,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A46,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A46,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A46,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A46,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A46,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A46,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G46" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A46,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A46,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A46,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A46,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A46,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A46,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A46,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A46,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A46,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A46,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A46,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A46,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A46,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A46,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A46,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A46,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A46,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A46,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A46,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9898,19 +9919,19 @@
         <v/>
       </c>
       <c r="D47" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A47,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A47,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A47,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A47,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A47,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A47,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A47,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A47,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E47" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A47,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A47,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A47,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A47,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A47,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A47,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A47,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A47,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F47" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A47,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A47,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A47,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A47,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A47,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A47,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A47,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A47,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G47" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A47,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A47,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A47,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A47,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A47,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A47,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A47,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A47,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A47,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A47,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A47,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A47,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A47,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A47,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A47,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A47,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A47,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A47,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A47,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9927,19 +9948,19 @@
         <v/>
       </c>
       <c r="D48" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A48,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A48,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A48,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A48,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A48,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A48,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A48,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A48,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E48" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A48,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A48,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A48,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A48,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A48,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A48,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A48,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A48,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F48" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A48,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A48,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A48,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A48,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A48,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A48,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A48,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A48,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G48" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A48,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A48,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A48,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A48,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A48,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A48,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A48,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A48,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A48,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A48,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A48,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A48,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A48,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A48,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A48,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A48,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A48,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A48,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A48,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9956,19 +9977,19 @@
         <v/>
       </c>
       <c r="D49" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A49,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A49,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A49,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A49,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A49,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A49,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A49,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A49,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E49" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A49,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A49,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A49,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A49,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A49,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A49,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A49,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A49,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F49" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A49,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A49,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A49,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A49,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A49,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A49,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A49,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A49,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G49" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A49,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A49,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A49,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A49,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A49,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A49,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A49,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A49,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A49,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A49,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A49,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A49,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A49,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A49,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A49,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A49,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A49,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A49,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A49,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -9985,19 +10006,19 @@
         <v/>
       </c>
       <c r="D50" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A50,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A50,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A50,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A50,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A50,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A50,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A50,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A50,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E50" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A50,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A50,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A50,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A50,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A50,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A50,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A50,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A50,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F50" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A50,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A50,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A50,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A50,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A50,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A50,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A50,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A50,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G50" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A50,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A50,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A50,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A50,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A50,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A50,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A50,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A50,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A50,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A50,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A50,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A50,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A50,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A50,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A50,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A50,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A50,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A50,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A50,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10014,19 +10035,19 @@
         <v/>
       </c>
       <c r="D51" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A51,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A51,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A51,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A51,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A51,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A51,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A51,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A51,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E51" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A51,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A51,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A51,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A51,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A51,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A51,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A51,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A51,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F51" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A51,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A51,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A51,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A51,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A51,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A51,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A51,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A51,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G51" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A51,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A51,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A51,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A51,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A51,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A51,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A51,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A51,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A51,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A51,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A51,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A51,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A51,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A51,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A51,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A51,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A51,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A51,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A51,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10043,19 +10064,19 @@
         <v/>
       </c>
       <c r="D52" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A52,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A52,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A52,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A52,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A52,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A52,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A52,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A52,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E52" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A52,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A52,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A52,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A52,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A52,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A52,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A52,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A52,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F52" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A52,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A52,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A52,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A52,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A52,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A52,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A52,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A52,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G52" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A52,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A52,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A52,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A52,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A52,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A52,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A52,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A52,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A52,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A52,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A52,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A52,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A52,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A52,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A52,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A52,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A52,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A52,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A52,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10072,19 +10093,19 @@
         <v/>
       </c>
       <c r="D53" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A53,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A53,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A53,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A53,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A53,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A53,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A53,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A53,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E53" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A53,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A53,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A53,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A53,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A53,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A53,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A53,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A53,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F53" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A53,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A53,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A53,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A53,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A53,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A53,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A53,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A53,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G53" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A53,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A53,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A53,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A53,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A53,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A53,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A53,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A53,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A53,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A53,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A53,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A53,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A53,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A53,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A53,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A53,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A53,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A53,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A53,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10101,19 +10122,19 @@
         <v/>
       </c>
       <c r="D54" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A54,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A54,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A54,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A54,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A54,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A54,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A54,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A54,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E54" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A54,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A54,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A54,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A54,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A54,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A54,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A54,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A54,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F54" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A54,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A54,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A54,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A54,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A54,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A54,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A54,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A54,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G54" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A54,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A54,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A54,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A54,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A54,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A54,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A54,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A54,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A54,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A54,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A54,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A54,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A54,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A54,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A54,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A54,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A54,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A54,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A54,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10130,19 +10151,19 @@
         <v/>
       </c>
       <c r="D55" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A55,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A55,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A55,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A55,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A55,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A55,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A55,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A55,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E55" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A55,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A55,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A55,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A55,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A55,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A55,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A55,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A55,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F55" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A55,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A55,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A55,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A55,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A55,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A55,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A55,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A55,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G55" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A55,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A55,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A55,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A55,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A55,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A55,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A55,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A55,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A55,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A55,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A55,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A55,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A55,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A55,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A55,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A55,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A55,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A55,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A55,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10159,19 +10180,19 @@
         <v/>
       </c>
       <c r="D56" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A56,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A56,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A56,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A56,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A56,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A56,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A56,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A56,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E56" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A56,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A56,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A56,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A56,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A56,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A56,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A56,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A56,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F56" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A56,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A56,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A56,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A56,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A56,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A56,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A56,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A56,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G56" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A56,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A56,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A56,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A56,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A56,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A56,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A56,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A56,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A56,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A56,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A56,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A56,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A56,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A56,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A56,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A56,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A56,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A56,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A56,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10188,19 +10209,19 @@
         <v/>
       </c>
       <c r="D57" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A57,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A57,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A57,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A57,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A57,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A57,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A57,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A57,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E57" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A57,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A57,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A57,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A57,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A57,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A57,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A57,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A57,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F57" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A57,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A57,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A57,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A57,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A57,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A57,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A57,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A57,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G57" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A57,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A57,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A57,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A57,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A57,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A57,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A57,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A57,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A57,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A57,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A57,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A57,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A57,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A57,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A57,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A57,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A57,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A57,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A57,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10217,19 +10238,19 @@
         <v/>
       </c>
       <c r="D58" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A58,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A58,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A58,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A58,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A58,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A58,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A58,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A58,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E58" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A58,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A58,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A58,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A58,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A58,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A58,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A58,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A58,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F58" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A58,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A58,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A58,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A58,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A58,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A58,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A58,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A58,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G58" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A58,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A58,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A58,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A58,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A58,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A58,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A58,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A58,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A58,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A58,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A58,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A58,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A58,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A58,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A58,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A58,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A58,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A58,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A58,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10246,19 +10267,19 @@
         <v/>
       </c>
       <c r="D59" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A59,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A59,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A59,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A59,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A59,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A59,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A59,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A59,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E59" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A59,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A59,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A59,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A59,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A59,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A59,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A59,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A59,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F59" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A59,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A59,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A59,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A59,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A59,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A59,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A59,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A59,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G59" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A59,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A59,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A59,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A59,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A59,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A59,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A59,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A59,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A59,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A59,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A59,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A59,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A59,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A59,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A59,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A59,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A59,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A59,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A59,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10275,19 +10296,19 @@
         <v/>
       </c>
       <c r="D60" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A60,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A60,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A60,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A60,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A60,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A60,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A60,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A60,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E60" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A60,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A60,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A60,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A60,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A60,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A60,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A60,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A60,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F60" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A60,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A60,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A60,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A60,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A60,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A60,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A60,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A60,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G60" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A60,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A60,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A60,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A60,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A60,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A60,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A60,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A60,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A60,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A60,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A60,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A60,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A60,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A60,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A60,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A60,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A60,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A60,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A60,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10304,19 +10325,19 @@
         <v/>
       </c>
       <c r="D61" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A61,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A61,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A61,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A61,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A61,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A61,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A61,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A61,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E61" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A61,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A61,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A61,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A61,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A61,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A61,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A61,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A61,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F61" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A61,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A61,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A61,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A61,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A61,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A61,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A61,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A61,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G61" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A61,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A61,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A61,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A61,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A61,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A61,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A61,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A61,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A61,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A61,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A61,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A61,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A61,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A61,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A61,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A61,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A61,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A61,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A61,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10333,19 +10354,19 @@
         <v/>
       </c>
       <c r="D62" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A62,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A62,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A62,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A62,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A62,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A62,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A62,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A62,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E62" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A62,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A62,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A62,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A62,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A62,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A62,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A62,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A62,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F62" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A62,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A62,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A62,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A62,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A62,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A62,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A62,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A62,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G62" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A62,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A62,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A62,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A62,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A62,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A62,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A62,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A62,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A62,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A62,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A62,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A62,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A62,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A62,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A62,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A62,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A62,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A62,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A62,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10362,19 +10383,19 @@
         <v/>
       </c>
       <c r="D63" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A63,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A63,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A63,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A63,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A63,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A63,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A63,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A63,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E63" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A63,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A63,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A63,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A63,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A63,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A63,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A63,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A63,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F63" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A63,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A63,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A63,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A63,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A63,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A63,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A63,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A63,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G63" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A63,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A63,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A63,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A63,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A63,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A63,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A63,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A63,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A63,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A63,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A63,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A63,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A63,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A63,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A63,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A63,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A63,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A63,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A63,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10391,19 +10412,19 @@
         <v/>
       </c>
       <c r="D64" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A64,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A64,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A64,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A64,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A64,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A64,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A64,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A64,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E64" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A64,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A64,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A64,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A64,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A64,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A64,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A64,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A64,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F64" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A64,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A64,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A64,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A64,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A64,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A64,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A64,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A64,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G64" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A64,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A64,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A64,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A64,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A64,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A64,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A64,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A64,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A64,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A64,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A64,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A64,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A64,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A64,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A64,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A64,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A64,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A64,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A64,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10420,19 +10441,19 @@
         <v/>
       </c>
       <c r="D65" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A65,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A65,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A65,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A65,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A65,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A65,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A65,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A65,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E65" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A65,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A65,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A65,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A65,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A65,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A65,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A65,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A65,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F65" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A65,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A65,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A65,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A65,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A65,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A65,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A65,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A65,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G65" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A65,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A65,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A65,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A65,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A65,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A65,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A65,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A65,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A65,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A65,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A65,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A65,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A65,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A65,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A65,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A65,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A65,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A65,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A65,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10449,19 +10470,19 @@
         <v/>
       </c>
       <c r="D66" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A66,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A66,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A66,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A66,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A66,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A66,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A66,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A66,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E66" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A66,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A66,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A66,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A66,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A66,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A66,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A66,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A66,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F66" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A66,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A66,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A66,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A66,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A66,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A66,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A66,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A66,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G66" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A66,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A66,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A66,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A66,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A66,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A66,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A66,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A66,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A66,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A66,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A66,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A66,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A66,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A66,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A66,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A66,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A66,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A66,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A66,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10478,19 +10499,19 @@
         <v/>
       </c>
       <c r="D67" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A67,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A67,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A67,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A67,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A67,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A67,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A67,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A67,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E67" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A67,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A67,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A67,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A67,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A67,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A67,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A67,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A67,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F67" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A67,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A67,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A67,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A67,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A67,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A67,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A67,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A67,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G67" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A67,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A67,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A67,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A67,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A67,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A67,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A67,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A67,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A67,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A67,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A67,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A67,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A67,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A67,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A67,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A67,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A67,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A67,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A67,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10507,19 +10528,19 @@
         <v/>
       </c>
       <c r="D68" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A68,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A68,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A68,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A68,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A68,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A68,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A68,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A68,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E68" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A68,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A68,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A68,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A68,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A68,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A68,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A68,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A68,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F68" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A68,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A68,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A68,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A68,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A68,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A68,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A68,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A68,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G68" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A68,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A68,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A68,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A68,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A68,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A68,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A68,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A68,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A68,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A68,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A68,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A68,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A68,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A68,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A68,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A68,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A68,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A68,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A68,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10536,19 +10557,19 @@
         <v/>
       </c>
       <c r="D69" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A69,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A69,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A69,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A69,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A69,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A69,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A69,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A69,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E69" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A69,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A69,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A69,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A69,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A69,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A69,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A69,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A69,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F69" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A69,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A69,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A69,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A69,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A69,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A69,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A69,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A69,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G69" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A69,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A69,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A69,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A69,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A69,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A69,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A69,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A69,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A69,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A69,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A69,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A69,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A69,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A69,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A69,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A69,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A69,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A69,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A69,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10565,19 +10586,19 @@
         <v/>
       </c>
       <c r="D70" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A70,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A70,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A70,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A70,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A70,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A70,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A70,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A70,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E70" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A70,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A70,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A70,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A70,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A70,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A70,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A70,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A70,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F70" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A70,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A70,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A70,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A70,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A70,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A70,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A70,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A70,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G70" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A70,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A70,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A70,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A70,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A70,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A70,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A70,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A70,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A70,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A70,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A70,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A70,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A70,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A70,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A70,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A70,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A70,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A70,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A70,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10594,19 +10615,19 @@
         <v/>
       </c>
       <c r="D71" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A71,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A71,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A71,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A71,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A71,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A71,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A71,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A71,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E71" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A71,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A71,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A71,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A71,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A71,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A71,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A71,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A71,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F71" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A71,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A71,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A71,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A71,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A71,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A71,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A71,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A71,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G71" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A71,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A71,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A71,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A71,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A71,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A71,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A71,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A71,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A71,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A71,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A71,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A71,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A71,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A71,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A71,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A71,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A71,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A71,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A71,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10623,19 +10644,19 @@
         <v/>
       </c>
       <c r="D72" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A72,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A72,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A72,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A72,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A72,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A72,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A72,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A72,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E72" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A72,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A72,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A72,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A72,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A72,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A72,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A72,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A72,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F72" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A72,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A72,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A72,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A72,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A72,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A72,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A72,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A72,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G72" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A72,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A72,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A72,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A72,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A72,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A72,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A72,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A72,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A72,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A72,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A72,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A72,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A72,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A72,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A72,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A72,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A72,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A72,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A72,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10652,19 +10673,19 @@
         <v/>
       </c>
       <c r="D73" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A73,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A73,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A73,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A73,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A73,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A73,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A73,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A73,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E73" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A73,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A73,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A73,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A73,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A73,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A73,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A73,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A73,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F73" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A73,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A73,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A73,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A73,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A73,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A73,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A73,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A73,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G73" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A73,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A73,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A73,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A73,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A73,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A73,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A73,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A73,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A73,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A73,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A73,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A73,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A73,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A73,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A73,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A73,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A73,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A73,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A73,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10681,19 +10702,19 @@
         <v/>
       </c>
       <c r="D74" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A74,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A74,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A74,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A74,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A74,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A74,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A74,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A74,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E74" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A74,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A74,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A74,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A74,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A74,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A74,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A74,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A74,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F74" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A74,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A74,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A74,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A74,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A74,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A74,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A74,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A74,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G74" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A74,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A74,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A74,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A74,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A74,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A74,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A74,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A74,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A74,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A74,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A74,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A74,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A74,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A74,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A74,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A74,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A74,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A74,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A74,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10710,19 +10731,19 @@
         <v/>
       </c>
       <c r="D75" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A75,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A75,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A75,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A75,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A75,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A75,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A75,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A75,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E75" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A75,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A75,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A75,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A75,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A75,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A75,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A75,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A75,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F75" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A75,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A75,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A75,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A75,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A75,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A75,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A75,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A75,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G75" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A75,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A75,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A75,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A75,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A75,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A75,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A75,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A75,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A75,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A75,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A75,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A75,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A75,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A75,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A75,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A75,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A75,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A75,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A75,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10739,19 +10760,19 @@
         <v/>
       </c>
       <c r="D76" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A76,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A76,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A76,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A76,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A76,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A76,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A76,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A76,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E76" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A76,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A76,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A76,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A76,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A76,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A76,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A76,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A76,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F76" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A76,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A76,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A76,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A76,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A76,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A76,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A76,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A76,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G76" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A76,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A76,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A76,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A76,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A76,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A76,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A76,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A76,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A76,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A76,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A76,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A76,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A76,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A76,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A76,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A76,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A76,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A76,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A76,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10768,19 +10789,19 @@
         <v/>
       </c>
       <c r="D77" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A77,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A77,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A77,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A77,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A77,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A77,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A77,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A77,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E77" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A77,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A77,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A77,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A77,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A77,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A77,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A77,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A77,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F77" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A77,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A77,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A77,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A77,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A77,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A77,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A77,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A77,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G77" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A77,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A77,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A77,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A77,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A77,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A77,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A77,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A77,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A77,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A77,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A77,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A77,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A77,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A77,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A77,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A77,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A77,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A77,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A77,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10797,19 +10818,19 @@
         <v/>
       </c>
       <c r="D78" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A78,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A78,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A78,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A78,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A78,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A78,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A78,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A78,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E78" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A78,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A78,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A78,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A78,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A78,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A78,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A78,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A78,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F78" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A78,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A78,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A78,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A78,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A78,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A78,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A78,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A78,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G78" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A78,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A78,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A78,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A78,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A78,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A78,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A78,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A78,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A78,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A78,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A78,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A78,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A78,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A78,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A78,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A78,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A78,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A78,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A78,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10826,19 +10847,19 @@
         <v/>
       </c>
       <c r="D79" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A79,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A79,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A79,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A79,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A79,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A79,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A79,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A79,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E79" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A79,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A79,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A79,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A79,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A79,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A79,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A79,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A79,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F79" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A79,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A79,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A79,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A79,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A79,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A79,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A79,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A79,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G79" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A79,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A79,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A79,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A79,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A79,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A79,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A79,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A79,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A79,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A79,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A79,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A79,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A79,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A79,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A79,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A79,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A79,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A79,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A79,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10855,19 +10876,19 @@
         <v/>
       </c>
       <c r="D80" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A80,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A80,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A80,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A80,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A80,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A80,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A80,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A80,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E80" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A80,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A80,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A80,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A80,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A80,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A80,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A80,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A80,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F80" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A80,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A80,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A80,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A80,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A80,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A80,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A80,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A80,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G80" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A80,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A80,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A80,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A80,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A80,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A80,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A80,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A80,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A80,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A80,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A80,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A80,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A80,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A80,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A80,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A80,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A80,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A80,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A80,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10884,19 +10905,19 @@
         <v/>
       </c>
       <c r="D81" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A81,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A81,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A81,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A81,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A81,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A81,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A81,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A81,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E81" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A81,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A81,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A81,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A81,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A81,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A81,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A81,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A81,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F81" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A81,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A81,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A81,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A81,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A81,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A81,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A81,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A81,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G81" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A81,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A81,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A81,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A81,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A81,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A81,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A81,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A81,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A81,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A81,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A81,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A81,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A81,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A81,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A81,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A81,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A81,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A81,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A81,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10913,19 +10934,19 @@
         <v/>
       </c>
       <c r="D82" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A82,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A82,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A82,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A82,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A82,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A82,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A82,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A82,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E82" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A82,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A82,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A82,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A82,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A82,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A82,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A82,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A82,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F82" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A82,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A82,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A82,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A82,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A82,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A82,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A82,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A82,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G82" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A82,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A82,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A82,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A82,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A82,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A82,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A82,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A82,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A82,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A82,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A82,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A82,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A82,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A82,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A82,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A82,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A82,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A82,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A82,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10942,19 +10963,19 @@
         <v/>
       </c>
       <c r="D83" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A83,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A83,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A83,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A83,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A83,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A83,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A83,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A83,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E83" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A83,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A83,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A83,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A83,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A83,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A83,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A83,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A83,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F83" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A83,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A83,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A83,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A83,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A83,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A83,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A83,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A83,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G83" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A83,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A83,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A83,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A83,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A83,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A83,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A83,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A83,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A83,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A83,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A83,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A83,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A83,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A83,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A83,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A83,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A83,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A83,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A83,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -10971,19 +10992,19 @@
         <v/>
       </c>
       <c r="D84" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A84,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A84,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A84,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A84,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A84,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A84,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A84,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A84,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E84" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A84,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A84,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A84,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A84,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A84,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A84,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A84,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A84,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F84" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A84,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A84,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A84,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A84,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A84,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A84,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A84,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A84,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G84" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A84,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A84,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A84,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A84,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A84,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A84,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A84,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A84,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A84,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A84,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A84,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A84,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A84,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A84,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A84,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A84,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A84,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A84,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A84,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11000,19 +11021,19 @@
         <v/>
       </c>
       <c r="D85" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A85,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A85,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A85,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A85,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A85,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A85,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A85,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A85,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E85" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A85,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A85,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A85,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A85,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A85,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A85,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A85,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A85,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F85" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A85,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A85,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A85,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A85,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A85,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A85,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A85,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A85,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G85" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A85,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A85,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A85,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A85,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A85,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A85,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A85,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A85,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A85,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A85,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A85,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A85,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A85,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A85,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A85,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A85,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A85,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A85,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A85,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11029,19 +11050,19 @@
         <v/>
       </c>
       <c r="D86" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A86,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A86,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A86,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A86,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A86,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A86,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A86,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A86,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E86" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A86,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A86,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A86,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A86,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A86,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A86,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A86,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A86,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F86" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A86,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A86,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A86,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A86,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A86,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A86,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A86,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A86,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G86" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A86,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A86,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A86,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A86,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A86,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A86,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A86,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A86,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A86,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A86,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A86,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A86,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A86,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A86,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A86,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A86,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A86,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A86,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A86,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11058,19 +11079,19 @@
         <v/>
       </c>
       <c r="D87" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A87,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A87,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A87,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A87,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A87,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A87,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A87,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A87,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E87" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A87,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A87,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A87,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A87,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A87,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A87,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A87,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A87,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F87" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A87,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A87,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A87,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A87,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A87,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A87,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A87,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A87,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G87" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A87,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A87,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A87,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A87,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A87,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A87,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A87,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A87,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A87,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A87,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A87,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A87,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A87,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A87,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A87,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A87,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A87,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A87,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A87,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11087,19 +11108,19 @@
         <v/>
       </c>
       <c r="D88" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A88,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A88,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A88,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A88,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A88,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A88,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A88,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A88,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E88" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A88,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A88,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A88,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A88,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A88,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A88,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A88,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A88,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F88" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A88,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A88,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A88,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A88,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A88,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A88,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A88,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A88,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G88" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A88,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A88,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A88,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A88,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A88,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A88,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A88,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A88,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A88,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A88,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A88,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A88,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A88,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A88,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A88,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A88,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A88,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A88,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A88,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11116,19 +11137,19 @@
         <v/>
       </c>
       <c r="D89" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A89,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A89,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A89,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A89,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A89,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A89,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A89,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A89,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E89" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A89,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A89,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A89,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A89,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A89,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A89,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A89,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A89,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F89" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A89,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A89,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A89,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A89,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A89,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A89,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A89,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A89,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G89" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A89,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A89,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A89,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A89,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A89,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A89,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A89,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A89,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A89,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A89,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A89,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A89,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A89,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A89,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A89,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A89,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A89,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A89,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A89,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11145,19 +11166,19 @@
         <v/>
       </c>
       <c r="D90" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A90,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A90,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A90,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A90,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A90,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A90,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A90,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A90,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E90" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A90,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A90,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A90,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A90,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A90,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A90,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A90,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A90,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F90" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A90,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A90,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A90,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A90,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A90,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A90,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A90,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A90,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G90" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A90,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A90,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A90,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A90,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A90,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A90,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A90,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A90,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A90,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A90,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A90,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A90,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A90,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A90,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A90,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A90,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A90,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A90,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A90,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11174,19 +11195,19 @@
         <v/>
       </c>
       <c r="D91" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A91,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A91,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A91,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A91,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A91,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A91,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A91,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A91,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E91" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A91,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A91,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A91,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A91,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A91,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A91,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A91,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A91,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F91" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A91,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A91,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A91,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A91,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A91,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A91,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A91,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A91,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G91" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A91,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A91,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A91,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A91,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A91,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A91,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A91,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A91,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A91,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A91,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A91,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A91,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A91,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A91,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A91,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A91,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A91,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A91,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A91,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11203,19 +11224,19 @@
         <v/>
       </c>
       <c r="D92" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A92,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A92,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A92,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A92,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A92,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A92,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A92,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A92,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E92" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A92,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A92,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A92,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A92,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A92,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A92,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A92,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A92,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F92" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A92,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A92,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A92,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A92,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A92,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A92,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A92,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A92,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G92" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A92,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A92,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A92,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A92,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A92,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A92,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A92,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A92,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A92,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A92,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A92,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A92,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A92,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A92,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A92,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A92,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A92,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A92,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A92,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11232,19 +11253,19 @@
         <v/>
       </c>
       <c r="D93" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A93,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A93,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A93,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A93,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A93,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A93,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A93,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A93,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E93" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A93,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A93,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A93,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A93,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A93,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A93,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A93,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A93,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F93" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A93,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A93,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A93,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A93,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A93,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A93,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A93,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A93,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G93" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A93,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A93,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A93,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A93,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A93,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A93,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A93,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A93,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A93,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A93,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A93,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A93,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A93,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A93,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A93,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A93,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A93,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A93,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A93,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11261,19 +11282,19 @@
         <v/>
       </c>
       <c r="D94" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A94,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A94,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A94,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A94,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A94,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A94,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A94,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A94,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E94" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A94,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A94,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A94,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A94,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A94,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A94,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A94,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A94,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F94" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A94,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A94,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A94,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A94,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A94,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A94,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A94,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A94,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G94" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A94,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A94,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A94,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A94,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A94,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A94,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A94,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A94,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A94,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A94,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A94,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A94,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A94,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A94,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A94,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A94,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A94,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A94,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A94,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11290,19 +11311,19 @@
         <v/>
       </c>
       <c r="D95" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A95,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A95,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A95,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A95,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A95,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A95,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A95,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A95,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E95" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A95,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A95,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A95,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A95,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A95,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A95,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A95,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A95,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F95" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A95,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A95,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A95,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A95,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A95,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A95,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A95,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A95,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G95" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A95,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A95,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A95,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A95,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A95,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A95,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A95,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A95,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A95,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A95,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A95,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A95,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A95,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A95,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A95,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A95,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A95,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A95,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A95,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11319,19 +11340,19 @@
         <v/>
       </c>
       <c r="D96" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A96,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A96,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A96,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A96,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A96,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A96,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A96,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A96,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E96" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A96,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A96,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A96,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A96,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A96,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A96,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A96,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A96,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F96" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A96,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A96,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A96,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A96,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A96,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A96,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A96,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A96,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G96" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A96,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A96,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A96,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A96,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A96,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A96,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A96,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A96,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A96,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A96,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A96,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A96,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A96,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A96,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A96,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A96,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A96,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A96,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A96,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11348,19 +11369,19 @@
         <v/>
       </c>
       <c r="D97" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A97,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A97,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A97,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A97,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A97,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A97,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A97,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A97,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E97" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A97,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A97,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A97,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A97,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A97,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A97,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A97,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A97,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F97" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A97,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A97,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A97,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A97,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A97,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A97,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A97,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A97,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G97" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A97,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A97,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A97,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A97,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A97,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A97,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A97,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A97,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A97,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A97,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A97,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A97,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A97,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A97,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A97,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A97,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A97,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A97,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A97,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11377,19 +11398,19 @@
         <v/>
       </c>
       <c r="D98" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A98,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A98,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A98,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A98,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A98,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A98,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A98,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A98,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E98" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A98,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A98,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A98,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A98,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A98,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A98,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A98,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A98,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F98" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A98,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A98,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A98,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A98,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A98,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A98,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A98,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A98,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G98" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A98,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A98,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A98,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A98,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A98,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A98,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A98,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A98,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A98,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A98,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A98,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A98,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A98,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A98,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A98,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A98,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A98,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A98,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A98,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11406,19 +11427,19 @@
         <v/>
       </c>
       <c r="D99" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A99,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A99,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A99,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A99,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A99,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A99,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A99,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A99,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E99" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A99,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A99,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A99,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A99,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A99,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A99,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A99,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A99,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F99" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A99,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A99,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A99,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A99,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A99,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A99,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A99,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A99,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G99" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A99,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A99,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A99,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A99,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A99,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A99,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A99,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A99,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A99,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A99,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A99,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A99,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A99,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A99,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A99,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A99,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A99,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A99,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A99,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11435,19 +11456,19 @@
         <v/>
       </c>
       <c r="D100" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A100,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A100,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A100,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A100,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A100,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A100,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A100,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A100,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E100" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A100,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A100,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A100,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A100,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A100,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A100,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A100,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A100,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F100" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A100,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A100,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A100,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A100,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A100,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A100,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A100,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A100,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G100" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A100,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A100,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A100,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A100,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A100,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A100,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A100,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A100,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A100,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A100,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A100,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A100,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A100,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A100,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A100,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A100,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A100,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A100,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A100,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11464,19 +11485,19 @@
         <v/>
       </c>
       <c r="D101" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A101,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A101,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A101,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A101,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A101,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A101,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A101,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A101,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E101" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A101,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A101,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A101,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A101,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A101,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A101,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A101,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A101,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F101" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A101,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A101,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A101,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A101,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A101,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A101,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A101,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A101,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G101" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A101,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A101,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A101,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A101,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A101,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A101,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A101,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A101,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A101,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A101,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A101,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A101,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A101,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A101,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A101,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A101,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A101,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A101,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A101,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11493,19 +11514,19 @@
         <v/>
       </c>
       <c r="D102" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A102,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A102,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A102,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A102,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A102,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A102,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A102,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A102,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E102" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A102,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A102,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A102,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A102,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A102,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A102,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A102,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A102,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F102" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A102,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A102,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A102,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A102,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A102,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A102,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A102,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A102,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G102" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A102,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A102,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A102,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A102,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A102,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A102,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A102,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A102,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A102,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A102,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A102,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A102,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A102,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A102,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A102,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A102,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A102,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A102,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A102,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11522,19 +11543,19 @@
         <v/>
       </c>
       <c r="D103" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A103,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A103,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A103,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A103,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A103,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A103,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A103,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A103,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E103" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A103,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A103,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A103,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A103,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A103,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A103,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A103,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A103,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F103" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A103,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A103,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A103,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A103,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A103,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A103,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A103,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A103,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G103" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A103,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A103,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A103,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A103,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A103,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A103,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A103,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A103,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A103,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A103,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A103,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A103,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A103,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A103,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A103,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A103,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A103,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A103,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A103,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11551,19 +11572,19 @@
         <v/>
       </c>
       <c r="D104" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A104,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A104,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A104,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A104,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A104,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A104,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A104,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A104,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E104" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A104,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A104,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A104,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A104,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A104,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A104,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A104,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A104,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F104" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A104,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A104,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A104,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A104,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A104,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A104,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A104,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A104,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G104" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A104,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A104,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A104,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A104,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A104,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A104,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A104,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A104,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A104,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A104,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A104,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A104,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A104,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A104,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A104,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A104,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A104,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A104,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A104,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11580,19 +11601,19 @@
         <v/>
       </c>
       <c r="D105" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A105,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A105,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A105,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A105,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A105,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A105,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A105,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A105,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E105" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A105,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A105,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A105,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A105,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A105,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A105,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A105,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A105,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F105" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A105,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A105,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A105,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A105,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A105,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A105,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A105,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A105,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G105" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A105,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A105,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A105,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A105,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A105,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A105,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A105,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A105,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A105,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A105,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A105,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A105,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A105,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A105,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A105,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A105,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A105,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A105,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A105,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11609,19 +11630,19 @@
         <v/>
       </c>
       <c r="D106" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A106,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A106,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A106,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A106,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A106,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A106,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A106,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A106,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E106" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A106,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A106,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A106,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A106,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A106,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A106,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A106,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A106,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F106" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A106,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A106,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A106,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A106,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A106,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A106,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A106,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A106,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G106" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A106,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A106,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A106,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A106,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A106,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A106,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A106,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A106,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A106,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A106,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A106,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A106,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A106,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A106,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A106,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A106,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A106,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A106,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A106,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11638,19 +11659,19 @@
         <v/>
       </c>
       <c r="D107" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A107,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A107,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A107,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A107,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A107,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A107,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A107,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A107,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E107" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A107,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A107,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A107,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A107,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A107,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A107,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A107,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A107,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F107" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A107,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A107,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A107,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A107,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A107,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A107,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A107,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A107,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G107" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A107,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A107,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A107,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A107,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A107,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A107,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A107,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A107,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A107,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A107,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A107,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A107,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A107,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A107,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A107,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A107,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A107,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A107,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A107,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11667,19 +11688,19 @@
         <v/>
       </c>
       <c r="D108" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A108,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A108,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A108,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A108,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A108,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A108,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A108,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A108,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E108" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A108,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A108,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A108,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A108,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A108,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A108,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A108,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A108,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F108" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A108,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A108,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A108,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A108,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A108,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A108,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A108,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A108,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G108" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A108,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A108,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A108,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A108,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A108,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A108,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A108,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A108,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A108,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A108,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A108,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A108,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A108,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A108,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A108,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A108,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A108,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A108,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A108,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11696,19 +11717,19 @@
         <v/>
       </c>
       <c r="D109" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A109,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A109,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A109,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A109,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A109,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A109,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A109,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A109,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E109" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A109,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A109,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A109,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A109,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A109,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A109,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A109,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A109,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F109" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A109,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A109,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A109,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A109,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A109,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A109,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A109,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A109,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G109" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A109,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A109,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A109,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A109,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A109,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A109,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A109,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A109,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A109,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A109,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A109,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A109,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A109,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A109,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A109,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A109,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A109,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A109,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A109,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11725,19 +11746,19 @@
         <v/>
       </c>
       <c r="D110" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A110,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A110,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A110,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A110,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A110,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A110,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A110,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A110,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E110" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A110,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A110,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A110,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A110,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A110,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A110,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A110,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A110,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F110" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A110,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A110,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A110,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A110,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A110,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A110,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A110,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A110,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G110" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A110,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A110,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A110,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A110,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A110,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A110,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A110,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A110,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A110,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A110,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A110,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A110,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A110,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A110,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A110,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A110,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A110,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A110,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A110,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11754,19 +11775,19 @@
         <v/>
       </c>
       <c r="D111" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A111,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A111,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A111,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A111,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A111,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A111,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A111,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A111,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E111" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A111,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A111,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A111,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A111,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A111,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A111,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A111,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A111,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F111" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A111,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A111,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A111,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A111,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A111,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A111,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A111,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A111,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G111" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A111,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A111,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A111,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A111,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A111,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A111,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A111,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A111,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A111,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A111,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A111,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A111,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A111,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A111,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A111,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A111,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A111,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A111,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A111,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11783,19 +11804,19 @@
         <v/>
       </c>
       <c r="D112" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A112,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A112,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A112,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A112,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A112,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A112,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A112,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A112,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E112" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A112,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A112,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A112,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A112,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A112,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A112,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A112,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A112,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F112" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A112,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A112,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A112,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A112,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A112,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A112,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A112,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A112,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G112" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A112,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A112,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A112,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A112,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A112,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A112,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A112,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A112,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A112,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A112,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A112,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A112,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A112,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A112,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A112,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A112,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A112,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A112,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A112,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11812,19 +11833,19 @@
         <v/>
       </c>
       <c r="D113" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A113,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A113,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A113,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A113,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A113,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A113,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A113,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A113,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E113" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A113,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A113,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A113,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A113,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A113,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A113,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A113,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A113,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F113" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A113,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A113,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A113,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A113,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A113,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A113,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A113,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A113,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G113" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A113,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A113,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A113,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A113,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A113,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A113,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A113,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A113,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A113,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A113,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A113,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A113,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A113,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A113,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A113,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A113,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A113,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A113,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A113,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11841,19 +11862,19 @@
         <v/>
       </c>
       <c r="D114" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A114,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A114,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A114,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A114,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A114,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A114,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A114,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A114,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E114" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A114,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A114,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A114,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A114,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A114,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A114,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A114,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A114,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F114" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A114,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A114,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A114,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A114,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A114,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A114,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A114,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A114,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G114" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A114,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A114,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A114,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A114,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A114,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A114,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A114,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A114,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A114,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A114,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A114,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A114,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A114,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A114,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A114,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A114,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A114,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A114,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A114,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11870,19 +11891,19 @@
         <v/>
       </c>
       <c r="D115" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A115,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A115,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A115,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A115,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A115,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A115,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A115,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A115,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E115" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A115,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A115,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A115,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A115,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A115,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A115,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A115,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A115,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F115" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A115,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A115,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A115,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A115,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A115,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A115,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A115,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A115,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G115" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A115,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A115,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A115,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A115,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A115,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A115,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A115,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A115,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A115,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A115,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A115,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A115,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A115,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A115,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A115,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A115,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A115,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A115,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A115,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11899,19 +11920,19 @@
         <v/>
       </c>
       <c r="D116" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A116,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A116,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A116,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A116,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A116,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A116,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A116,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A116,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E116" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A116,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A116,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A116,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A116,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A116,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A116,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A116,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A116,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F116" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A116,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A116,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A116,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A116,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A116,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A116,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A116,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A116,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G116" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A116,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A116,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A116,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A116,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A116,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A116,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A116,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A116,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A116,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A116,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A116,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A116,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A116,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A116,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A116,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A116,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A116,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A116,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A116,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11928,19 +11949,19 @@
         <v/>
       </c>
       <c r="D117" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A117,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A117,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A117,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A117,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A117,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A117,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A117,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A117,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E117" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A117,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A117,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A117,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A117,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A117,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A117,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A117,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A117,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F117" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A117,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A117,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A117,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A117,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A117,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A117,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A117,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A117,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G117" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A117,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A117,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A117,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A117,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A117,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A117,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A117,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A117,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A117,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A117,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A117,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A117,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A117,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A117,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A117,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A117,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A117,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A117,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A117,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11957,19 +11978,19 @@
         <v/>
       </c>
       <c r="D118" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A118,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A118,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A118,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A118,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A118,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A118,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A118,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A118,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E118" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A118,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A118,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A118,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A118,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A118,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A118,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A118,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A118,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F118" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A118,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A118,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A118,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A118,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A118,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A118,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A118,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A118,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G118" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A118,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A118,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A118,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A118,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A118,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A118,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A118,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A118,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A118,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A118,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A118,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A118,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A118,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A118,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A118,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A118,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A118,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A118,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A118,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -11986,19 +12007,19 @@
         <v/>
       </c>
       <c r="D119" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A119,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A119,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A119,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A119,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A119,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A119,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A119,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A119,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E119" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A119,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A119,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A119,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A119,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A119,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A119,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A119,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A119,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F119" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A119,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A119,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A119,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A119,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A119,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A119,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A119,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A119,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G119" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A119,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A119,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A119,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A119,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A119,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A119,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A119,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A119,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A119,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A119,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A119,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A119,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A119,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A119,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A119,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A119,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A119,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A119,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A119,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -12015,19 +12036,19 @@
         <v/>
       </c>
       <c r="D120" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A120,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A120,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A120,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A120,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A120,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A120,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A120,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A120,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E120" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A120,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A120,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A120,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A120,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A120,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A120,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A120,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A120,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F120" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A120,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A120,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A120,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A120,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A120,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A120,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A120,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A120,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G120" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A120,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A120,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A120,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A120,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A120,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A120,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A120,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A120,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A120,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A120,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A120,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A120,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A120,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A120,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A120,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A120,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A120,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A120,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A120,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -12044,19 +12065,19 @@
         <v/>
       </c>
       <c r="D121" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A121,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A121,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A121,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A121,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A121,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A121,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A121,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A121,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E121" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A121,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A121,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A121,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A121,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A121,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A121,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A121,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A121,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F121" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A121,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A121,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A121,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A121,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A121,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A121,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A121,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A121,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G121" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A121,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A121,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A121,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A121,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A121,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A121,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A121,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A121,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A121,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A121,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A121,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A121,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A121,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A121,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A121,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A121,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A121,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A121,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A121,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -12073,19 +12094,19 @@
         <v/>
       </c>
       <c r="D122" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A122,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A122,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A122,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A122,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A122,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A122,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A122,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A122,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E122" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A122,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A122,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A122,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A122,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A122,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A122,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A122,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A122,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F122" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A122,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A122,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A122,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A122,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A122,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A122,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A122,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A122,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G122" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A122,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A122,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A122,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A122,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A122,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A122,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A122,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A122,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A122,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A122,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A122,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A122,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A122,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A122,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A122,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A122,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A122,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A122,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A122,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -12102,19 +12123,19 @@
         <v/>
       </c>
       <c r="D123" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A123,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A123,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A123,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A123,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A123,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A123,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A123,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A123,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E123" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A123,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A123,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A123,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A123,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A123,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A123,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A123,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A123,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F123" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A123,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A123,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A123,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A123,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A123,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A123,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A123,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A123,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G123" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A123,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A123,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A123,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A123,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A123,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A123,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A123,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A123,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A123,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A123,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A123,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A123,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A123,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A123,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A123,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A123,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A123,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A123,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A123,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -12131,19 +12152,19 @@
         <v/>
       </c>
       <c r="D124" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A124,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A124,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A124,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A124,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A124,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A124,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A124,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A124,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E124" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A124,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A124,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A124,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A124,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A124,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A124,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A124,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A124,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F124" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A124,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A124,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A124,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A124,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A124,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A124,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A124,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A124,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G124" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A124,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A124,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A124,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A124,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A124,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A124,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A124,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A124,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A124,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A124,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A124,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A124,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A124,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A124,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A124,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A124,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A124,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A124,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A124,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -12160,19 +12181,19 @@
         <v/>
       </c>
       <c r="D125" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A125,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A125,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A125,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A125,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A125,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A125,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A125,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A125,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E125" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A125,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A125,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A125,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A125,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A125,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A125,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A125,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A125,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F125" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A125,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A125,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A125,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A125,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A125,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A125,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A125,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A125,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G125" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A125,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A125,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A125,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A125,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A125,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A125,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A125,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A125,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A125,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A125,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A125,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A125,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A125,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A125,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A125,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A125,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A125,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A125,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A125,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -12189,19 +12210,19 @@
         <v/>
       </c>
       <c r="D126" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A126,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A126,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A126,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A126,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A126,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A126,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A126,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A126,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E126" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A126,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A126,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A126,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A126,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A126,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A126,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A126,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A126,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F126" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A126,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A126,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A126,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A126,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A126,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A126,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A126,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A126,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G126" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A126,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A126,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A126,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A126,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A126,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A126,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A126,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A126,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A126,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A126,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A126,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A126,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A126,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A126,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A126,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A126,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A126,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A126,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A126,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -12218,19 +12239,19 @@
         <v/>
       </c>
       <c r="D127" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A127,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A127,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A127,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A127,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A127,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A127,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A127,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A127,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E127" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A127,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A127,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A127,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A127,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A127,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A127,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A127,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A127,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F127" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A127,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A127,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A127,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A127,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A127,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A127,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A127,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A127,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G127" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A127,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A127,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A127,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A127,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A127,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A127,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A127,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A127,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A127,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A127,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A127,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A127,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A127,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A127,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A127,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A127,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A127,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A127,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A127,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -12247,19 +12268,19 @@
         <v/>
       </c>
       <c r="D128" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A128,'S3'!$E$6:$E$19,"Víctor")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A128,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A128,'S4'!$E$6:$E$20,"Víctor")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A128,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Víctor")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Víctor")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A128,'S3'!$E$6:$E$24,"Víctor")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A128,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A128,'S4'!$E$6:$E$22,"Víctor")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A128,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Víctor")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Víctor")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Víctor")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Víctor")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Víctor")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Víctor")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Víctor")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Víctor")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Víctor")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="E128" s="21">
-        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A128,'S3'!$E$6:$E$19,"Diego")+SUMIFS('S3'!$I$6:$I$19,'S3'!$B$6:$B$19,$A128,'S3'!$E$6:$E$19,"Ambos")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A128,'S4'!$E$6:$E$20,"Diego")+SUMIFS('S4'!$I$6:$I$20,'S4'!$B$6:$B$20,$A128,'S4'!$E$6:$E$20,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Diego")+SUMIFS('S1'!$I$6:$I$32,'S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Ambos")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Diego")+SUMIFS('S2'!$I$6:$I$23,'S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Ambos")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A128,'S3'!$E$6:$E$24,"Diego")+SUMIFS('S3'!$I$6:$I$24,'S3'!$B$6:$B$24,$A128,'S3'!$E$6:$E$24,"Ambos")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A128,'S4'!$E$6:$E$22,"Diego")+SUMIFS('S4'!$I$6:$I$22,'S4'!$B$6:$B$22,$A128,'S4'!$E$6:$E$22,"Ambos")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Diego")+SUMIFS('S5'!$I$6:$I$20,'S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Ambos")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Diego")+SUMIFS('S6'!$I$6:$I$17,'S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Ambos")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Diego")+SUMIFS('S7'!$I$6:$I$19,'S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Ambos")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Diego")+SUMIFS('S8'!$I$6:$I$23,'S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Ambos")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Diego")+SUMIFS('S9'!$I$6:$I$15,'S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Ambos")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Diego")+SUMIFS('S10'!$I$6:$I$13,'S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Ambos")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Diego")+SUMIFS('Holgura'!$I$6:$I$11,'Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Ambos")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Diego")+SUMIFS('Entrega'!$I$6:$I$9,'Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Ambos")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Diego")+SUMIFS('Defensa'!$I$6:$I$10,'Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="F128" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A128,'S3'!$E$6:$E$19,"Víctor")+COUNTIFS('S3'!$B$6:$B$19,$A128,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A128,'S4'!$E$6:$E$20,"Víctor")+COUNTIFS('S4'!$B$6:$B$20,$A128,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Víctor")+COUNTIFS('S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Víctor")+COUNTIFS('S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A128,'S3'!$E$6:$E$24,"Víctor")+COUNTIFS('S3'!$B$6:$B$24,$A128,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A128,'S4'!$E$6:$E$22,"Víctor")+COUNTIFS('S4'!$B$6:$B$22,$A128,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Víctor")+COUNTIFS('S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Víctor")+COUNTIFS('S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Víctor")+COUNTIFS('S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Víctor")+COUNTIFS('S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Víctor")+COUNTIFS('S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Víctor")+COUNTIFS('S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Víctor")+COUNTIFS('Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Víctor")+COUNTIFS('Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Víctor")+COUNTIFS('Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
       <c r="G128" s="21">
-        <f>COUNTIFS('S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$19,$A128,'S3'!$E$6:$E$19,"Diego")+COUNTIFS('S3'!$B$6:$B$19,$A128,'S3'!$E$6:$E$19,"Ambos")+COUNTIFS('S4'!$B$6:$B$20,$A128,'S4'!$E$6:$E$20,"Diego")+COUNTIFS('S4'!$B$6:$B$20,$A128,'S4'!$E$6:$E$20,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Ambos")</f>
+        <f>COUNTIFS('S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Diego")+COUNTIFS('S1'!$B$6:$B$32,$A128,'S1'!$E$6:$E$32,"Ambos")+COUNTIFS('S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Diego")+COUNTIFS('S2'!$B$6:$B$23,$A128,'S2'!$E$6:$E$23,"Ambos")+COUNTIFS('S3'!$B$6:$B$24,$A128,'S3'!$E$6:$E$24,"Diego")+COUNTIFS('S3'!$B$6:$B$24,$A128,'S3'!$E$6:$E$24,"Ambos")+COUNTIFS('S4'!$B$6:$B$22,$A128,'S4'!$E$6:$E$22,"Diego")+COUNTIFS('S4'!$B$6:$B$22,$A128,'S4'!$E$6:$E$22,"Ambos")+COUNTIFS('S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Diego")+COUNTIFS('S5'!$B$6:$B$20,$A128,'S5'!$E$6:$E$20,"Ambos")+COUNTIFS('S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Diego")+COUNTIFS('S6'!$B$6:$B$17,$A128,'S6'!$E$6:$E$17,"Ambos")+COUNTIFS('S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Diego")+COUNTIFS('S7'!$B$6:$B$19,$A128,'S7'!$E$6:$E$19,"Ambos")+COUNTIFS('S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Diego")+COUNTIFS('S8'!$B$6:$B$23,$A128,'S8'!$E$6:$E$23,"Ambos")+COUNTIFS('S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Diego")+COUNTIFS('S9'!$B$6:$B$15,$A128,'S9'!$E$6:$E$15,"Ambos")+COUNTIFS('S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Diego")+COUNTIFS('S10'!$B$6:$B$13,$A128,'S10'!$E$6:$E$13,"Ambos")+COUNTIFS('Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Diego")+COUNTIFS('Holgura'!$B$6:$B$11,$A128,'Holgura'!$E$6:$E$11,"Ambos")+COUNTIFS('Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Diego")+COUNTIFS('Entrega'!$B$6:$B$9,$A128,'Entrega'!$E$6:$E$9,"Ambos")+COUNTIFS('Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Diego")+COUNTIFS('Defensa'!$B$6:$B$10,$A128,'Defensa'!$E$6:$E$10,"Ambos")</f>
         <v/>
       </c>
     </row>
@@ -12543,7 +12564,7 @@
       <c r="J7" s="22" t="n"/>
       <c r="K7" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Movido</t>
         </is>
       </c>
       <c r="L7" s="15">
@@ -12557,7 +12578,7 @@
       </c>
       <c r="N7" s="15" t="inlineStr">
         <is>
-          <t>Depende del campo. Mientras tanto Diego sigue con lo movido del S1 (IA_DIEGO.md)</t>
+          <t>Depende del campo. Mientras tanto Diego sigue con lo movido del S1 (IA_DIEGO.md) · 27-oct: bloqueada, no hay datos de campo; copia en S4-T17 (reprogramada 27-oct)</t>
         </is>
       </c>
     </row>
@@ -12669,7 +12690,7 @@
       <c r="J9" s="22" t="n"/>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Movido</t>
         </is>
       </c>
       <c r="L9" s="15">
@@ -12683,7 +12704,7 @@
       </c>
       <c r="N9" s="15" t="inlineStr">
         <is>
-          <t>Depende del campo</t>
+          <t>Depende del campo · 27-oct: bloqueada, no hay datos de campo; copia en S4-T17 (reprogramada 27-oct)</t>
         </is>
       </c>
     </row>
@@ -12792,10 +12813,12 @@
       <c r="I11" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="J11" s="22" t="n"/>
+      <c r="J11" s="22" t="n">
+        <v>46320</v>
+      </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L11" s="15">
@@ -12809,7 +12832,7 @@
       </c>
       <c r="N11" s="15" t="inlineStr">
         <is>
-          <t>Empezar el borrador con los documentos que hay (informe final del 22-jul y diagnóstico) y completarlo con las entrevistas cuando haya campo</t>
+          <t>Empezar el borrador con los documentos que hay (informe final del 22-jul y diagnóstico) y completarlo con las entrevistas cuando haya campo · 25-oct: AS-IS v0.1 (.bpmn, .png y .md) con el Informe Final del 22-jul; borrador sin validar en campo</t>
         </is>
       </c>
     </row>
@@ -12918,10 +12941,12 @@
       <c r="I13" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="J13" s="22" t="n"/>
+      <c r="J13" s="22" t="n">
+        <v>46320</v>
+      </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L13" s="15">
@@ -12933,7 +12958,11 @@
           <t>S2-05 (#17)</t>
         </is>
       </c>
-      <c r="N13" s="15" t="inlineStr"/>
+      <c r="N13" s="15" t="inlineStr">
+        <is>
+          <t>25-oct: 5 puntos donde se pierde tiempo marcados; la validación con entrevistas queda para el campo</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
@@ -13104,10 +13133,12 @@
       <c r="I16" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="J16" s="22" t="n"/>
+      <c r="J16" s="22" t="n">
+        <v>46320</v>
+      </c>
       <c r="K16" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L16" s="15">
@@ -13119,7 +13150,11 @@
           <t>S2-06 (#18)</t>
         </is>
       </c>
-      <c r="N16" s="15" t="inlineStr"/>
+      <c r="N16" s="15" t="inlineStr">
+        <is>
+          <t>25-oct: 07_Flujos_Diseno/2026-10-25_Inventario_Herramientas_v0.1.xlsx (13 herramientas, criterios C1–C8)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
@@ -13288,10 +13323,12 @@
       <c r="I19" s="24" t="n">
         <v>2.5</v>
       </c>
-      <c r="J19" s="22" t="n"/>
+      <c r="J19" s="22" t="n">
+        <v>46320</v>
+      </c>
       <c r="K19" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="L19" s="15">
@@ -13303,7 +13340,11 @@
           <t>S2-06 (#18)</t>
         </is>
       </c>
-      <c r="N19" s="15" t="inlineStr"/>
+      <c r="N19" s="15" t="inlineStr">
+        <is>
+          <t>25-oct: inventario v0.2 con pesos y puntuación</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
@@ -13349,7 +13390,7 @@
       <c r="J20" s="22" t="n"/>
       <c r="K20" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Movido</t>
         </is>
       </c>
       <c r="L20" s="15">
@@ -13361,7 +13402,11 @@
           <t>S2-05 (#17)</t>
         </is>
       </c>
-      <c r="N20" s="15" t="inlineStr"/>
+      <c r="N20" s="15" t="inlineStr">
+        <is>
+          <t>27-oct: la descripción está en 2026-10-25_AS-IS_v0.1.md, pero falta el resumen de 1 página; copia en S3-T19 (reprogramada 27-oct)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
@@ -13471,7 +13516,7 @@
       <c r="J22" s="22" t="n"/>
       <c r="K22" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Movido</t>
         </is>
       </c>
       <c r="L22" s="15">
@@ -13483,7 +13528,11 @@
           <t>S2-04 (#16)</t>
         </is>
       </c>
-      <c r="N22" s="15" t="inlineStr"/>
+      <c r="N22" s="15" t="inlineStr">
+        <is>
+          <t>27-oct: bloqueada, sin datos; en la Revisión 1 se muestra el AS-IS; copia en S4-T17 (reprogramada 27-oct)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
@@ -13529,7 +13578,7 @@
       <c r="J23" s="22" t="n"/>
       <c r="K23" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Movido</t>
         </is>
       </c>
       <c r="L23" s="15">
@@ -13541,7 +13590,11 @@
           <t>S2-08 (#59)</t>
         </is>
       </c>
-      <c r="N23" s="15" t="inlineStr"/>
+      <c r="N23" s="15" t="inlineStr">
+        <is>
+          <t>27-oct: revisión escrita en la bitácora; la llamada con Diego se hace junto con el ensayo (S3-T03, reprogramada 27-oct)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A5:N23"/>
@@ -13577,7 +13630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -13643,11 +13696,11 @@
         </is>
       </c>
       <c r="C3" s="12">
-        <f>IFERROR(COUNTIF(K6:K19,"Hecho")/(COUNTA(D6:D19)-COUNTIF(K6:K19,"Cancelado")),0)</f>
+        <f>IFERROR(COUNTIF(K6:K24,"Hecho")/(COUNTA(D6:D24)-COUNTIF(K6:K24,"Cancelado")),0)</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>"Víctor: "&amp;TEXT(IFERROR((COUNTIFS(E6:E19,"Víctor",K6:K19,"Hecho")+COUNTIFS(E6:E19,"Ambos",K6:K19,"Hecho"))/(COUNTIF(E6:E19,"Víctor")+COUNTIF(E6:E19,"Ambos")),0),"0%")&amp;"   ·   Diego: "&amp;TEXT(IFERROR((COUNTIFS(E6:E19,"Diego",K6:K19,"Hecho")+COUNTIFS(E6:E19,"Ambos",K6:K19,"Hecho"))/(COUNTIF(E6:E19,"Diego")+COUNTIF(E6:E19,"Ambos")),0),"0%")&amp;"   ·   Horas: "&amp;TEXT(SUM(I6:I19),"0.0")</f>
+        <f>"Víctor: "&amp;TEXT(IFERROR((COUNTIFS(E6:E24,"Víctor",K6:K24,"Hecho")+COUNTIFS(E6:E24,"Ambos",K6:K24,"Hecho"))/(COUNTIF(E6:E24,"Víctor")+COUNTIF(E6:E24,"Ambos")),0),"0%")&amp;"   ·   Diego: "&amp;TEXT(IFERROR((COUNTIFS(E6:E24,"Diego",K6:K24,"Hecho")+COUNTIFS(E6:E24,"Ambos",K6:K24,"Hecho"))/(COUNTIF(E6:E24,"Diego")+COUNTIF(E6:E24,"Ambos")),0),"0%")&amp;"   ·   Horas: "&amp;TEXT(SUM(I6:I24),"0.0")</f>
         <v/>
       </c>
     </row>
@@ -13825,7 +13878,7 @@
       <c r="J7" s="22" t="n"/>
       <c r="K7" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="L7" s="15">
@@ -13837,7 +13890,11 @@
           <t>S3-03 (#21)</t>
         </is>
       </c>
-      <c r="N7" s="15" t="inlineStr"/>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>27-oct: la figura ya existe (07_Flujos_Diseno/2026-10-25_AS-IS_v0.1.png); no hay gráficas de datos porque no hay campo</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
@@ -13895,7 +13952,11 @@
           <t>S3-01 (#19)</t>
         </is>
       </c>
-      <c r="N8" s="15" t="inlineStr"/>
+      <c r="N8" s="15" t="inlineStr">
+        <is>
+          <t>27-oct en la noche; incluye la revisión del sprint 2 que quedó pendiente (S2-T18)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
@@ -14539,8 +14600,318 @@
       </c>
       <c r="N19" s="15" t="inlineStr"/>
     </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>S3-T15</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="n">
+        <v>46322</v>
+      </c>
+      <c r="C20" s="23">
+        <f>B20</f>
+        <v/>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>Confirmar si TEAMSLASH guarda los datos en Google Sheets o en PostgreSQL, para el documento de elicitación</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="inlineStr">
+        <is>
+          <t>Diego</t>
+        </is>
+      </c>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>WhatsApp a Víctor · repositorio de TEAMSLASH</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>Respuesta con evidencia (captura o enlace)</t>
+        </is>
+      </c>
+      <c r="H20" s="15" t="inlineStr">
+        <is>
+          <t>Víctor tiene la respuesta</t>
+        </is>
+      </c>
+      <c r="I20" s="24" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J20" s="22" t="n"/>
+      <c r="K20" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L20" s="15">
+        <f>IF(K20="Cancelado","",IF(J20&lt;&gt;"",J20-B20,IF(AND(K20&lt;&gt;"Hecho",TODAY()&gt;B20),TODAY()-B20,0)))</f>
+        <v/>
+      </c>
+      <c r="M20" s="15" t="inlineStr">
+        <is>
+          <t>S4-04 (#25)</t>
+        </is>
+      </c>
+      <c r="N20" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente desde el 20-oct (reprogramada 27-oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>S3-T16</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="n">
+        <v>46323</v>
+      </c>
+      <c r="C21" s="23">
+        <f>B21</f>
+        <v/>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>Conseguir la respuesta de Torvesa (autorización de campo, nota de respaldo y catálogo), para medir la línea base</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>Diego</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>Torvesa (llamada o visita al Ing. Torres)</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>Autorización por escrito o fecha de campo comprometida</t>
+        </is>
+      </c>
+      <c r="H21" s="15" t="inlineStr">
+        <is>
+          <t>Víctor tiene la respuesta y la fecha del campo</t>
+        </is>
+      </c>
+      <c r="I21" s="24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J21" s="22" t="n"/>
+      <c r="K21" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L21" s="15">
+        <f>IF(K21="Cancelado","",IF(J21&lt;&gt;"",J21-B21,IF(AND(K21&lt;&gt;"Hecho",TODAY()&gt;B21),TODAY()-B21,0)))</f>
+        <v/>
+      </c>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>S1-09 (#9)</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>Riesgo principal. Si no hay respuesta el 30-oct: pedir carta de respaldo a la tutora (reprogramada 27-oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>S3-T17</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="n">
+        <v>46325</v>
+      </c>
+      <c r="C22" s="23">
+        <f>B22</f>
+        <v/>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>Revisar y completar la elicitación y análisis de requerimientos v0.1, parte 1: requerimientos técnicos (no funcionales y restricciones) y TEAMSLASH</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>Diego</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>07_Flujos_Diseno/2026-10-27_Elicitacion_Requerimientos_v0.1.docx (Word, control de cambios)</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>Cambios y comentarios de Diego en el Word</t>
+        </is>
+      </c>
+      <c r="H22" s="15" t="inlineStr">
+        <is>
+          <t>Cada requerimiento técnico con criterio de aceptación y fuente</t>
+        </is>
+      </c>
+      <c r="I22" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="22" t="n"/>
+      <c r="K22" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L22" s="15">
+        <f>IF(K22="Cancelado","",IF(J22&lt;&gt;"",J22-B22,IF(AND(K22&lt;&gt;"Hecho",TODAY()&gt;B22),TODAY()-B22,0)))</f>
+        <v/>
+      </c>
+      <c r="M22" s="15" t="inlineStr">
+        <is>
+          <t>S4-04 (#25)</t>
+        </is>
+      </c>
+      <c r="N22" s="15" t="inlineStr">
+        <is>
+          <t>Tarea nueva (27-oct). Claude saca la v0.2 con lo que marque Diego</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>S3-T18</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="n">
+        <v>46326</v>
+      </c>
+      <c r="C23" s="23">
+        <f>B23</f>
+        <v/>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>Completar la elicitación v0.1, parte 2: diagrama de casos de uso y modelo conceptual</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>Diego</t>
+        </is>
+      </c>
+      <c r="F23" s="15" t="inlineStr">
+        <is>
+          <t>07_Flujos_Diseno/ (editable en draw.io, demo.bpmn.io o Mermaid)</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>Casos de uso y modelo conceptual en PNG + archivo editable</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="inlineStr">
+        <is>
+          <t>Cada caso de uso enlazado a un escenario ESC-xx</t>
+        </is>
+      </c>
+      <c r="I23" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J23" s="22" t="n"/>
+      <c r="K23" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L23" s="15">
+        <f>IF(K23="Cancelado","",IF(J23&lt;&gt;"",J23-B23,IF(AND(K23&lt;&gt;"Hecho",TODAY()&gt;B23),TODAY()-B23,0)))</f>
+        <v/>
+      </c>
+      <c r="M23" s="15" t="inlineStr">
+        <is>
+          <t>S4-04 (#25)</t>
+        </is>
+      </c>
+      <c r="N23" s="15" t="inlineStr">
+        <is>
+          <t>Tarea nueva (27-oct). Va al anexo E del documento de elicitación</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>S3-T19</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="n">
+        <v>46327</v>
+      </c>
+      <c r="C24" s="23">
+        <f>B24</f>
+        <v/>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>Escribir el resumen de 1 página del proceso actual (AS-IS) para Víctor</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>Diego</t>
+        </is>
+      </c>
+      <c r="F24" s="15" t="inlineStr">
+        <is>
+          <t>07_Flujos_Diseno/</t>
+        </is>
+      </c>
+      <c r="G24" s="15" t="inlineStr">
+        <is>
+          <t>07_Flujos_Diseno/2026-11-01_Resumen_AS-IS.md</t>
+        </is>
+      </c>
+      <c r="H24" s="15" t="inlineStr">
+        <is>
+          <t>Víctor lo leyó</t>
+        </is>
+      </c>
+      <c r="I24" s="24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J24" s="22" t="n"/>
+      <c r="K24" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L24" s="15">
+        <f>IF(K24="Cancelado","",IF(J24&lt;&gt;"",J24-B24,IF(AND(K24&lt;&gt;"Hecho",TODAY()&gt;B24),TODAY()-B24,0)))</f>
+        <v/>
+      </c>
+      <c r="M24" s="15" t="inlineStr">
+        <is>
+          <t>S2-05 (#17)</t>
+        </is>
+      </c>
+      <c r="N24" s="15" t="inlineStr">
+        <is>
+          <t>Copia de S2-T15 (reprogramada 27-oct)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:N19"/>
+  <autoFilter ref="A5:N24"/>
   <conditionalFormatting sqref="A6:N19">
     <cfRule type="expression" priority="1" dxfId="1" stopIfTrue="1">
       <formula>$K6="Hecho"</formula>
@@ -14553,6 +14924,20 @@
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="3">
       <formula>$K6="Cancelado"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A20:N24">
+    <cfRule type="expression" priority="5" dxfId="1" stopIfTrue="1">
+      <formula>$K20="Hecho"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="2" stopIfTrue="1">
+      <formula>$K20="Movido"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="1">
+      <formula>AND($K20&lt;&gt;"Cancelado",$L20&lt;&gt;"",$L20&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="3">
+      <formula>$K20="Cancelado"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -14573,7 +14958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -14639,11 +15024,11 @@
         </is>
       </c>
       <c r="C3" s="12">
-        <f>IFERROR(COUNTIF(K6:K20,"Hecho")/(COUNTA(D6:D20)-COUNTIF(K6:K20,"Cancelado")),0)</f>
+        <f>IFERROR(COUNTIF(K6:K22,"Hecho")/(COUNTA(D6:D22)-COUNTIF(K6:K22,"Cancelado")),0)</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>"Víctor: "&amp;TEXT(IFERROR((COUNTIFS(E6:E20,"Víctor",K6:K20,"Hecho")+COUNTIFS(E6:E20,"Ambos",K6:K20,"Hecho"))/(COUNTIF(E6:E20,"Víctor")+COUNTIF(E6:E20,"Ambos")),0),"0%")&amp;"   ·   Diego: "&amp;TEXT(IFERROR((COUNTIFS(E6:E20,"Diego",K6:K20,"Hecho")+COUNTIFS(E6:E20,"Ambos",K6:K20,"Hecho"))/(COUNTIF(E6:E20,"Diego")+COUNTIF(E6:E20,"Ambos")),0),"0%")&amp;"   ·   Horas: "&amp;TEXT(SUM(I6:I20),"0.0")</f>
+        <f>"Víctor: "&amp;TEXT(IFERROR((COUNTIFS(E6:E22,"Víctor",K6:K22,"Hecho")+COUNTIFS(E6:E22,"Ambos",K6:K22,"Hecho"))/(COUNTIF(E6:E22,"Víctor")+COUNTIF(E6:E22,"Ambos")),0),"0%")&amp;"   ·   Diego: "&amp;TEXT(IFERROR((COUNTIFS(E6:E22,"Diego",K6:K22,"Hecho")+COUNTIFS(E6:E22,"Ambos",K6:K22,"Hecho"))/(COUNTIF(E6:E22,"Diego")+COUNTIF(E6:E22,"Ambos")),0),"0%")&amp;"   ·   Horas: "&amp;TEXT(SUM(I6:I22),"0.0")</f>
         <v/>
       </c>
     </row>
@@ -15589,8 +15974,132 @@
       </c>
       <c r="N20" s="15" t="inlineStr"/>
     </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>S4-T16</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="n">
+        <v>46329</v>
+      </c>
+      <c r="C21" s="23">
+        <f>B21</f>
+        <v/>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>Hacer el campo en Torvesa (si autorizó): cronometrar cotizaciones (P2-A) y revisar solicitudes de los últimos 3 meses (P2-B)</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>Diego</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>Torvesa (oficina, Quito)</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>05_Datos_Campo/LineaBase_2026-10/P2A_cronometraje.csv y P2B_muestra_documental.csv</t>
+        </is>
+      </c>
+      <c r="H21" s="15" t="inlineStr">
+        <is>
+          <t>Todas las cotizaciones observables registradas</t>
+        </is>
+      </c>
+      <c r="I21" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="J21" s="22" t="n"/>
+      <c r="K21" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L21" s="15">
+        <f>IF(K21="Cancelado","",IF(J21&lt;&gt;"",J21-B21,IF(AND(K21&lt;&gt;"Hecho",TODAY()&gt;B21),TODAY()-B21,0)))</f>
+        <v/>
+      </c>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>S1-09 (#9)</t>
+        </is>
+      </c>
+      <c r="N21" s="15" t="inlineStr">
+        <is>
+          <t>Copia de S1-T16 y S1-T18 (reprogramada 27-oct). Solo si Torvesa autorizó. Día cargado: S4-T03 se termina el 8-nov si hace falta</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>S4-T17</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="n">
+        <v>46334</v>
+      </c>
+      <c r="C22" s="23">
+        <f>B22</f>
+        <v/>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>Analizar los datos de campo y preparar las gráficas de la línea base (M1–M4 y M6)</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>Diego</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>05_Datos_Campo/LineaBase_2026-10/</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>05_Datos_Campo/LineaBase_2026-10/analisis/ (Resultados_LineaBase_v0.1.md + figuras/)</t>
+        </is>
+      </c>
+      <c r="H22" s="15" t="inlineStr">
+        <is>
+          <t>Víctor entiende cada número</t>
+        </is>
+      </c>
+      <c r="I22" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J22" s="22" t="n"/>
+      <c r="K22" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L22" s="15">
+        <f>IF(K22="Cancelado","",IF(J22&lt;&gt;"",J22-B22,IF(AND(K22&lt;&gt;"Hecho",TODAY()&gt;B22),TODAY()-B22,0)))</f>
+        <v/>
+      </c>
+      <c r="M22" s="15" t="inlineStr">
+        <is>
+          <t>S2-04 (#16)</t>
+        </is>
+      </c>
+      <c r="N22" s="15" t="inlineStr">
+        <is>
+          <t>Copia de S2-T02, S2-T04 y S2-T17 (reprogramada 27-oct). Solo si hubo campo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:N20"/>
+  <autoFilter ref="A5:N22"/>
   <conditionalFormatting sqref="A6:N20">
     <cfRule type="expression" priority="1" dxfId="1" stopIfTrue="1">
       <formula>$K6="Hecho"</formula>
@@ -15603,6 +16112,20 @@
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="3">
       <formula>$K6="Cancelado"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A21:N22">
+    <cfRule type="expression" priority="5" dxfId="1" stopIfTrue="1">
+      <formula>$K21="Hecho"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="2" stopIfTrue="1">
+      <formula>$K21="Movido"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="1">
+      <formula>AND($K21&lt;&gt;"Cancelado",$L21&lt;&gt;"",$L21&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="3">
+      <formula>$K21="Cancelado"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">

</xml_diff>